<commit_message>
Atualização automática: reparaveis_rma (14/09/2026 09:27)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (14/09/2026 13:58)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (15/09/2026 08:57)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (15/09/2026 12:34)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (15/09/2026 14:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (16/09/2026 12:26)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (16/09/2026 12:43)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (17/09/2026 12:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (17/09/2026 12:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (18/09/2026 11:57)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (18/09/2026 16:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (21/09/2026 14:00)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (21/09/2026 14:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (22/09/2026 12:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (23/09/2026 10:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (23/09/2026 12:27)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (28/09/2026 13:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (28/09/2026 15:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (29/09/2026 19:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (30/09/2026 13:49)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,16 +5159,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5184,7 +5176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5192,30 +5184,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5515,52 +5489,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5775,7 +5749,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5912,7 +5886,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5953,7 +5927,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5988,7 +5962,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6029,7 +6003,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6067,7 +6041,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6108,7 +6082,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6149,7 +6123,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6187,7 +6161,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6228,7 +6202,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6269,7 +6243,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6310,7 +6284,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6351,7 +6325,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6453,7 +6427,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6494,7 +6468,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6535,7 +6509,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6576,7 +6550,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6617,7 +6591,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6658,7 +6632,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6731,7 +6705,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6804,7 +6778,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6845,7 +6819,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6886,7 +6860,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6927,7 +6901,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7000,7 +6974,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7105,7 +7079,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7146,7 +7120,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7187,7 +7161,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7228,7 +7202,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7269,7 +7243,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7310,7 +7284,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7348,7 +7322,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7389,7 +7363,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7430,7 +7404,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7503,7 +7477,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7544,7 +7518,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7617,7 +7591,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7690,7 +7664,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7763,7 +7737,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7833,7 +7807,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7906,7 +7880,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7941,7 +7915,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7982,7 +7956,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8023,7 +7997,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8064,7 +8038,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8105,7 +8079,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8146,7 +8120,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8187,7 +8161,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8228,7 +8202,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8263,7 +8237,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8304,7 +8278,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8342,7 +8316,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8380,7 +8354,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8418,7 +8392,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8456,7 +8430,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8497,7 +8471,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8538,7 +8512,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8579,7 +8553,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8620,7 +8594,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8661,7 +8635,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8702,7 +8676,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8743,7 +8717,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8784,7 +8758,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8863,7 +8837,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8904,7 +8878,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8945,7 +8919,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8986,7 +8960,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9027,7 +9001,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9068,7 +9042,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9109,7 +9083,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9150,7 +9124,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9223,7 +9197,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9264,7 +9238,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9305,7 +9279,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9346,7 +9320,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9387,7 +9361,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9425,7 +9399,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9495,7 +9469,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9536,7 +9510,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9577,7 +9551,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9618,7 +9592,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9720,7 +9694,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9761,7 +9735,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9802,7 +9776,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9843,7 +9817,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9881,7 +9855,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9919,7 +9893,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9960,7 +9934,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10001,7 +9975,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10042,7 +10016,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10083,7 +10057,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10124,7 +10098,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10165,7 +10139,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10206,7 +10180,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10247,7 +10221,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10285,7 +10259,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10326,7 +10300,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10367,7 +10341,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10437,7 +10411,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10510,7 +10484,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10551,7 +10525,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10592,7 +10566,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10665,7 +10639,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10706,7 +10680,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10747,7 +10721,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10785,7 +10759,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10858,7 +10832,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10896,7 +10870,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10966,7 +10940,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11071,7 +11045,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11112,7 +11086,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11153,7 +11127,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11194,7 +11168,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11235,7 +11209,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11276,7 +11250,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11317,7 +11291,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11390,7 +11364,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11431,7 +11405,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11472,7 +11446,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11513,7 +11487,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11583,7 +11557,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11624,7 +11598,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11665,7 +11639,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11706,7 +11680,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11747,7 +11721,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11788,7 +11762,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11826,7 +11800,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11899,7 +11873,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11940,7 +11914,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11978,7 +11952,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12013,7 +11987,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12054,7 +12028,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12095,7 +12069,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12174,7 +12148,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12215,7 +12189,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12256,7 +12230,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12297,7 +12271,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12338,7 +12312,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12379,7 +12353,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12420,7 +12394,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12461,7 +12435,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12534,7 +12508,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12601,7 +12575,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12674,7 +12648,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12715,7 +12689,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12756,7 +12730,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12797,7 +12771,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12838,7 +12812,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12879,7 +12853,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12952,7 +12926,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12993,7 +12967,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13034,7 +13008,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13075,7 +13049,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13116,7 +13090,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13157,7 +13131,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13195,7 +13169,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13236,7 +13210,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13315,7 +13289,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13356,7 +13330,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13397,7 +13371,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13438,7 +13412,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13476,7 +13450,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13517,7 +13491,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13558,7 +13532,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13596,7 +13570,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13637,7 +13611,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13678,7 +13652,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13719,7 +13693,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13833,7 +13807,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13874,7 +13848,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13915,7 +13889,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13956,7 +13930,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13997,7 +13971,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14358,7 +14332,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14399,7 +14373,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14440,7 +14414,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14481,7 +14455,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14522,7 +14496,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14563,7 +14537,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14604,7 +14578,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14741,7 +14715,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14782,7 +14756,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14855,7 +14829,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14896,7 +14870,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14934,7 +14908,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14972,7 +14946,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15234,7 +15208,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15380,7 +15354,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15421,7 +15395,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15462,7 +15436,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15500,7 +15474,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15541,7 +15515,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15582,7 +15556,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15623,7 +15597,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15667,7 +15641,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15708,7 +15682,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15749,7 +15723,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15790,7 +15764,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15831,7 +15805,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15875,7 +15849,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15910,7 +15884,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15948,7 +15922,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15983,7 +15957,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16024,7 +15998,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16062,7 +16036,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16103,7 +16077,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16141,7 +16115,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16179,7 +16153,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16217,7 +16191,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16255,7 +16229,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16296,7 +16270,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16334,7 +16308,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16375,7 +16349,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16416,7 +16390,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16521,7 +16495,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16562,7 +16536,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16603,7 +16577,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16644,7 +16618,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16685,7 +16659,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16726,7 +16700,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16767,7 +16741,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16808,7 +16782,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16849,7 +16823,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16884,7 +16858,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16919,7 +16893,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16954,7 +16928,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17027,7 +17001,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17068,7 +17042,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17109,7 +17083,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17150,7 +17124,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17188,7 +17162,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17229,7 +17203,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17270,7 +17244,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17311,7 +17285,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17352,7 +17326,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17393,7 +17367,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17434,7 +17408,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17475,7 +17449,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17516,7 +17490,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17551,7 +17525,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17592,7 +17566,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17633,7 +17607,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17674,7 +17648,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17715,7 +17689,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17756,7 +17730,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17797,7 +17771,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17838,7 +17812,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17943,7 +17917,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17984,7 +17958,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18121,7 +18095,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18191,7 +18165,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18232,7 +18206,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18264,7 +18238,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18305,7 +18279,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18343,7 +18317,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18381,7 +18355,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18419,7 +18393,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18454,7 +18428,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18492,7 +18466,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18530,7 +18504,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18568,7 +18542,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18606,7 +18580,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18644,7 +18618,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18682,7 +18656,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18720,7 +18694,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18761,7 +18735,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18866,7 +18840,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18971,7 +18945,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19009,7 +18983,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19079,7 +19053,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19114,7 +19088,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19152,7 +19126,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19196,7 +19170,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19231,7 +19205,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19269,7 +19243,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19345,7 +19319,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19383,7 +19357,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19453,7 +19427,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19494,7 +19468,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19532,7 +19506,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19570,7 +19544,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19614,7 +19588,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19652,7 +19626,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19693,7 +19667,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19734,7 +19708,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19775,7 +19749,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19941,7 +19915,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19982,7 +19956,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20023,7 +19997,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20064,7 +20038,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20105,7 +20079,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20146,7 +20120,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20187,7 +20161,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20228,7 +20202,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20269,7 +20243,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20342,7 +20316,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20572,7 +20546,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20613,7 +20587,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20654,7 +20628,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20727,7 +20701,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20765,7 +20739,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20803,7 +20777,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20870,7 +20844,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20943,7 +20917,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20984,7 +20958,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21025,7 +20999,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21066,7 +21040,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21133,7 +21107,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21174,7 +21148,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21212,7 +21186,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21250,7 +21224,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21285,7 +21259,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21422,7 +21396,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21457,7 +21431,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21492,7 +21466,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21559,7 +21533,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21600,7 +21574,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21641,7 +21615,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21682,7 +21656,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21720,7 +21694,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21761,7 +21735,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21802,7 +21776,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22000,7 +21974,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22041,7 +22015,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22254,7 +22228,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22295,7 +22269,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22333,7 +22307,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22374,7 +22348,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22415,7 +22389,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22450,7 +22424,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22485,7 +22459,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22552,7 +22526,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22593,7 +22567,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22628,7 +22602,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22663,7 +22637,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22736,7 +22710,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22777,7 +22751,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22815,7 +22789,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22850,7 +22824,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22949,7 +22923,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22993,7 +22967,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23060,7 +23034,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23159,7 +23133,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23200,7 +23174,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23241,7 +23215,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23282,7 +23256,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23320,7 +23294,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23358,7 +23332,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23396,7 +23370,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23437,7 +23411,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23475,7 +23449,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23513,7 +23487,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23551,7 +23525,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23624,7 +23598,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23796,7 +23770,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23837,7 +23811,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23878,7 +23852,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24143,7 +24117,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24184,7 +24158,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24333,7 +24307,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24374,7 +24348,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24412,7 +24386,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24488,7 +24462,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24532,7 +24506,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24573,7 +24547,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24678,7 +24652,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24722,7 +24696,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24798,7 +24772,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24833,7 +24807,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24874,7 +24848,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24909,7 +24883,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24950,7 +24924,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24991,7 +24965,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25032,7 +25006,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25073,7 +25047,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25178,7 +25152,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25312,7 +25286,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25449,7 +25423,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25586,7 +25560,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25691,7 +25665,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25729,7 +25703,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25930,7 +25904,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25974,7 +25948,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26009,7 +25983,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26044,7 +26018,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26242,7 +26216,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26347,7 +26321,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26388,7 +26362,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26554,7 +26528,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27372,7 +27346,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (05/10/2026 10:45)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5159,8 +5159,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5176,7 +5184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5184,12 +5192,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5489,52 +5515,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -5749,7 +5775,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -5886,7 +5912,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -5927,7 +5953,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -5962,7 +5988,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6003,7 +6029,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6041,7 +6067,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6082,7 +6108,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6123,7 +6149,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6161,7 +6187,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6202,7 +6228,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6243,7 +6269,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6284,7 +6310,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6325,7 +6351,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6427,7 +6453,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6468,7 +6494,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6509,7 +6535,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6550,7 +6576,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -6591,7 +6617,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -6632,7 +6658,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -6705,7 +6731,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -6778,7 +6804,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -6819,7 +6845,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -6860,7 +6886,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -6901,7 +6927,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -6974,7 +7000,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7079,7 +7105,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="2">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7120,7 +7146,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="2">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7161,7 +7187,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="2">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7202,7 +7228,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="2">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7243,7 +7269,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="2">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7284,7 +7310,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="2">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7322,7 +7348,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="2">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7363,7 +7389,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="2">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7404,7 +7430,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="2">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7477,7 +7503,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="2">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7518,7 +7544,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="2">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -7591,7 +7617,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="2">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -7664,7 +7690,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="2">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -7737,7 +7763,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="2">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -7807,7 +7833,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="2">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -7880,7 +7906,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="2">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -7915,7 +7941,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="2">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -7956,7 +7982,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="2">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -7997,7 +8023,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="2">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8038,7 +8064,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="2">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8079,7 +8105,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="2">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8120,7 +8146,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="2">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8161,7 +8187,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="2">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8202,7 +8228,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="2">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8237,7 +8263,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="2">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8278,7 +8304,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="2">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8316,7 +8342,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="2">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8354,7 +8380,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="2">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8392,7 +8418,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="2">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8430,7 +8456,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="2">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8471,7 +8497,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="2">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8512,7 +8538,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="2">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8553,7 +8579,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="2">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -8594,7 +8620,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="2">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -8635,7 +8661,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="2">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -8676,7 +8702,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="2">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -8717,7 +8743,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="2">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -8758,7 +8784,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="2">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -8837,7 +8863,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="2">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -8878,7 +8904,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="2">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -8919,7 +8945,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="2">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -8960,7 +8986,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="2">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9001,7 +9027,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="2">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9042,7 +9068,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="2">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9083,7 +9109,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="2">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9124,7 +9150,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="2">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9197,7 +9223,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="2">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9238,7 +9264,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="2">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9279,7 +9305,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="2">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9320,7 +9346,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="2">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9361,7 +9387,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="2">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9399,7 +9425,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="2">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9469,7 +9495,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="2">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9510,7 +9536,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="2">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9551,7 +9577,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="2">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -9592,7 +9618,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="2">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -9694,7 +9720,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="2">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -9735,7 +9761,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="2">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -9776,7 +9802,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="2">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -9817,7 +9843,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="2">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -9855,7 +9881,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="1">
+      <c r="D114" s="2">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -9893,7 +9919,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="1">
+      <c r="D115" s="2">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -9934,7 +9960,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="2">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -9975,7 +10001,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="1">
+      <c r="D117" s="2">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10016,7 +10042,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="1">
+      <c r="D118" s="2">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10057,7 +10083,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="1">
+      <c r="D119" s="2">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10098,7 +10124,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="1">
+      <c r="D120" s="2">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10139,7 +10165,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="1">
+      <c r="D121" s="2">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10180,7 +10206,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="1">
+      <c r="D122" s="2">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10221,7 +10247,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="1">
+      <c r="D123" s="2">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10259,7 +10285,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="1">
+      <c r="D124" s="2">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10300,7 +10326,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="1">
+      <c r="D125" s="2">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10341,7 +10367,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="1">
+      <c r="D126" s="2">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10411,7 +10437,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="1">
+      <c r="D128" s="2">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10484,7 +10510,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="1">
+      <c r="D130" s="2">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10525,7 +10551,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="1">
+      <c r="D131" s="2">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10566,7 +10592,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="1">
+      <c r="D132" s="2">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -10639,7 +10665,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="1">
+      <c r="D134" s="2">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -10680,7 +10706,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="1">
+      <c r="D135" s="2">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -10721,7 +10747,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="1">
+      <c r="D136" s="2">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -10759,7 +10785,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="1">
+      <c r="D137" s="2">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -10832,7 +10858,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="1">
+      <c r="D139" s="2">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -10870,7 +10896,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="1">
+      <c r="D140" s="2">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -10940,7 +10966,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="1">
+      <c r="D142" s="2">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11045,7 +11071,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="1">
+      <c r="D145" s="2">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11086,7 +11112,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="1">
+      <c r="D146" s="2">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11127,7 +11153,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="1">
+      <c r="D147" s="2">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11168,7 +11194,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="1">
+      <c r="D148" s="2">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11209,7 +11235,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="1">
+      <c r="D149" s="2">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11250,7 +11276,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="1">
+      <c r="D150" s="2">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11291,7 +11317,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="1">
+      <c r="D151" s="2">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11364,7 +11390,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="1">
+      <c r="D153" s="2">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11405,7 +11431,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D154" s="2">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11446,7 +11472,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D155" s="2">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11487,7 +11513,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="1">
+      <c r="D156" s="2">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11557,7 +11583,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="1">
+      <c r="D158" s="2">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -11598,7 +11624,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="1">
+      <c r="D159" s="2">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -11639,7 +11665,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="1">
+      <c r="D160" s="2">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -11680,7 +11706,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="1">
+      <c r="D161" s="2">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -11721,7 +11747,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="1">
+      <c r="D162" s="2">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -11762,7 +11788,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="1">
+      <c r="D163" s="2">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -11800,7 +11826,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="1">
+      <c r="D164" s="2">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -11873,7 +11899,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D166" s="2">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -11914,7 +11940,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="1">
+      <c r="D167" s="2">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -11952,7 +11978,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="1">
+      <c r="D168" s="2">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -11987,7 +12013,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="1">
+      <c r="D169" s="2">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12028,7 +12054,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="1">
+      <c r="D170" s="2">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12069,7 +12095,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="1">
+      <c r="D171" s="2">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12148,7 +12174,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="1">
+      <c r="D173" s="2">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12189,7 +12215,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="1">
+      <c r="D174" s="2">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12230,7 +12256,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D175" s="2">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12271,7 +12297,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="1">
+      <c r="D176" s="2">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12312,7 +12338,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="1">
+      <c r="D177" s="2">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12353,7 +12379,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="1">
+      <c r="D178" s="2">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12394,7 +12420,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="1">
+      <c r="D179" s="2">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12435,7 +12461,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="1">
+      <c r="D180" s="2">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12508,7 +12534,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="1">
+      <c r="D182" s="2">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -12575,7 +12601,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="1">
+      <c r="D184" s="2">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -12648,7 +12674,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="1">
+      <c r="D186" s="2">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -12689,7 +12715,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D187" s="2">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -12730,7 +12756,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="1">
+      <c r="D188" s="2">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -12771,7 +12797,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="1">
+      <c r="D189" s="2">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -12812,7 +12838,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="1">
+      <c r="D190" s="2">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -12853,7 +12879,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="1">
+      <c r="D191" s="2">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -12926,7 +12952,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="1">
+      <c r="D193" s="2">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -12967,7 +12993,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="1">
+      <c r="D194" s="2">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13008,7 +13034,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="1">
+      <c r="D195" s="2">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13049,7 +13075,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="1">
+      <c r="D196" s="2">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13090,7 +13116,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="1">
+      <c r="D197" s="2">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13131,7 +13157,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="1">
+      <c r="D198" s="2">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13169,7 +13195,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="1">
+      <c r="D199" s="2">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13210,7 +13236,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="1">
+      <c r="D200" s="2">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13289,7 +13315,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="1">
+      <c r="D202" s="2">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13330,7 +13356,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="1">
+      <c r="D203" s="2">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13371,7 +13397,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="1">
+      <c r="D204" s="2">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13412,7 +13438,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="1">
+      <c r="D205" s="2">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13450,7 +13476,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="1">
+      <c r="D206" s="2">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13491,7 +13517,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="1">
+      <c r="D207" s="2">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13532,7 +13558,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="1">
+      <c r="D208" s="2">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -13570,7 +13596,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="1">
+      <c r="D209" s="2">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -13611,7 +13637,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="1">
+      <c r="D210" s="2">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -13652,7 +13678,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="1">
+      <c r="D211" s="2">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -13693,7 +13719,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="1">
+      <c r="D212" s="2">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -13807,7 +13833,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="1">
+      <c r="D215" s="2">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -13848,7 +13874,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="1">
+      <c r="D216" s="2">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -13889,7 +13915,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="1">
+      <c r="D217" s="2">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -13930,7 +13956,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="1">
+      <c r="D218" s="2">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -13971,7 +13997,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="1">
+      <c r="D219" s="2">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14332,7 +14358,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="1">
+      <c r="D230" s="2">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14373,7 +14399,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="1">
+      <c r="D231" s="2">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14414,7 +14440,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="1">
+      <c r="D232" s="2">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14455,7 +14481,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="1">
+      <c r="D233" s="2">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14496,7 +14522,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="1">
+      <c r="D234" s="2">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14537,7 +14563,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="1">
+      <c r="D235" s="2">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -14578,7 +14604,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="1">
+      <c r="D236" s="2">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -14715,7 +14741,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="1">
+      <c r="D240" s="2">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -14756,7 +14782,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="1">
+      <c r="D241" s="2">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -14829,7 +14855,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="1">
+      <c r="D243" s="2">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -14870,7 +14896,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="1">
+      <c r="D244" s="2">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -14908,7 +14934,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="1">
+      <c r="D245" s="2">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -14946,7 +14972,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="1">
+      <c r="D246" s="2">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15208,7 +15234,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="1">
+      <c r="D254" s="2">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15313,7 +15339,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="1">
+      <c r="D257" s="2">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15354,7 +15380,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="1">
+      <c r="D258" s="2">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15395,7 +15421,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="1">
+      <c r="D259" s="2">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15436,7 +15462,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="1">
+      <c r="D260" s="2">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15474,7 +15500,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="1">
+      <c r="D261" s="2">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15515,7 +15541,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="1">
+      <c r="D262" s="2">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15556,7 +15582,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="1">
+      <c r="D263" s="2">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -15597,7 +15623,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="1">
+      <c r="D264" s="2">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -15641,7 +15667,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="1">
+      <c r="D265" s="2">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -15682,7 +15708,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="1">
+      <c r="D266" s="2">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -15723,7 +15749,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="1">
+      <c r="D267" s="2">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -15764,7 +15790,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="1">
+      <c r="D268" s="2">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -15805,7 +15831,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="1">
+      <c r="D269" s="2">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -15849,7 +15875,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="1">
+      <c r="D270" s="2">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -15884,7 +15910,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="1">
+      <c r="D271" s="2">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -15922,7 +15948,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="1">
+      <c r="D272" s="2">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -15957,7 +15983,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="1">
+      <c r="D273" s="2">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -15998,7 +16024,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="1">
+      <c r="D274" s="2">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16036,7 +16062,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="1">
+      <c r="D275" s="2">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16077,7 +16103,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="1">
+      <c r="D276" s="2">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16115,7 +16141,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="1">
+      <c r="D277" s="2">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16153,7 +16179,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="1">
+      <c r="D278" s="2">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16191,7 +16217,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="1">
+      <c r="D279" s="2">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16229,7 +16255,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="1">
+      <c r="D280" s="2">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16270,7 +16296,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="1">
+      <c r="D281" s="2">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16308,7 +16334,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="1">
+      <c r="D282" s="2">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16349,7 +16375,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="1">
+      <c r="D283" s="2">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16390,7 +16416,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="1">
+      <c r="D284" s="2">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16495,7 +16521,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="1">
+      <c r="D287" s="2">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16536,7 +16562,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="1">
+      <c r="D288" s="2">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -16577,7 +16603,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="1">
+      <c r="D289" s="2">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -16618,7 +16644,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="1">
+      <c r="D290" s="2">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -16659,7 +16685,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="1">
+      <c r="D291" s="2">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -16700,7 +16726,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="1">
+      <c r="D292" s="2">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -16741,7 +16767,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="1">
+      <c r="D293" s="2">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -16782,7 +16808,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="1">
+      <c r="D294" s="2">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -16823,7 +16849,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="1">
+      <c r="D295" s="2">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -16858,7 +16884,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="1">
+      <c r="D296" s="2">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -16893,7 +16919,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="1">
+      <c r="D297" s="2">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -16928,7 +16954,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="1">
+      <c r="D298" s="2">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17001,7 +17027,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="1">
+      <c r="D300" s="2">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17042,7 +17068,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="1">
+      <c r="D301" s="2">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17083,7 +17109,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="1">
+      <c r="D302" s="2">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17124,7 +17150,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="1">
+      <c r="D303" s="2">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17162,7 +17188,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="1">
+      <c r="D304" s="2">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17203,7 +17229,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="1">
+      <c r="D305" s="2">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17244,7 +17270,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="1">
+      <c r="D306" s="2">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17285,7 +17311,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="1">
+      <c r="D307" s="2">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17326,7 +17352,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="1">
+      <c r="D308" s="2">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17367,7 +17393,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="1">
+      <c r="D309" s="2">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17408,7 +17434,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="1">
+      <c r="D310" s="2">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17449,7 +17475,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="1">
+      <c r="D311" s="2">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17490,7 +17516,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="1">
+      <c r="D312" s="2">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17525,7 +17551,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="1">
+      <c r="D313" s="2">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17566,7 +17592,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="1">
+      <c r="D314" s="2">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -17607,7 +17633,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="1">
+      <c r="D315" s="2">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -17648,7 +17674,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="1">
+      <c r="D316" s="2">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -17689,7 +17715,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="1">
+      <c r="D317" s="2">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -17730,7 +17756,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="1">
+      <c r="D318" s="2">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -17771,7 +17797,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="1">
+      <c r="D319" s="2">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -17812,7 +17838,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="1">
+      <c r="D320" s="2">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -17917,7 +17943,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="1">
+      <c r="D323" s="2">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -17958,7 +17984,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="1">
+      <c r="D324" s="2">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18095,7 +18121,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="1">
+      <c r="D328" s="2">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18165,7 +18191,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="1">
+      <c r="D330" s="2">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18206,7 +18232,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="1">
+      <c r="D331" s="2">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18238,7 +18264,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="1">
+      <c r="D332" s="2">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18279,7 +18305,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="1">
+      <c r="D333" s="2">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18317,7 +18343,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="1">
+      <c r="D334" s="2">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18355,7 +18381,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="1">
+      <c r="D335" s="2">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18393,7 +18419,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="1">
+      <c r="D336" s="2">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18428,7 +18454,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="1">
+      <c r="D337" s="2">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18466,7 +18492,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="1">
+      <c r="D338" s="2">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18504,7 +18530,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="1">
+      <c r="D339" s="2">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18542,7 +18568,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="1">
+      <c r="D340" s="2">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -18580,7 +18606,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="1">
+      <c r="D341" s="2">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -18618,7 +18644,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="1">
+      <c r="D342" s="2">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -18656,7 +18682,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="1">
+      <c r="D343" s="2">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -18694,7 +18720,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="1">
+      <c r="D344" s="2">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -18735,7 +18761,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="1">
+      <c r="D345" s="2">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -18840,7 +18866,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="1">
+      <c r="D348" s="2">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -18945,7 +18971,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="1">
+      <c r="D351" s="2">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -18983,7 +19009,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="1">
+      <c r="D352" s="2">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19053,7 +19079,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="1">
+      <c r="D354" s="2">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19088,7 +19114,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="1">
+      <c r="D355" s="2">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19126,7 +19152,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="1">
+      <c r="D356" s="2">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19170,7 +19196,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="1">
+      <c r="D357" s="2">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19205,7 +19231,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="1">
+      <c r="D358" s="2">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19243,7 +19269,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="1">
+      <c r="D359" s="2">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19319,7 +19345,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="1">
+      <c r="D361" s="2">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19357,7 +19383,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="1">
+      <c r="D362" s="2">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19427,7 +19453,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="1">
+      <c r="D364" s="2">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19468,7 +19494,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="1">
+      <c r="D365" s="2">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19506,7 +19532,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="1">
+      <c r="D366" s="2">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19544,7 +19570,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="1">
+      <c r="D367" s="2">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -19588,7 +19614,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="1">
+      <c r="D368" s="2">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -19626,7 +19652,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="1">
+      <c r="D369" s="2">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -19667,7 +19693,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="1">
+      <c r="D370" s="2">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -19708,7 +19734,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="1">
+      <c r="D371" s="2">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -19749,7 +19775,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="1">
+      <c r="D372" s="2">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -19915,7 +19941,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="1">
+      <c r="D377" s="2">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -19956,7 +19982,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="1">
+      <c r="D378" s="2">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -19997,7 +20023,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="1">
+      <c r="D379" s="2">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20038,7 +20064,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="1">
+      <c r="D380" s="2">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20079,7 +20105,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="1">
+      <c r="D381" s="2">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20120,7 +20146,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="1">
+      <c r="D382" s="2">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20161,7 +20187,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="1">
+      <c r="D383" s="2">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20202,7 +20228,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="1">
+      <c r="D384" s="2">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20243,7 +20269,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="1">
+      <c r="D385" s="2">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20316,7 +20342,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="1">
+      <c r="D387" s="2">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20546,7 +20572,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="1">
+      <c r="D394" s="2">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -20587,7 +20613,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="1">
+      <c r="D395" s="2">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -20628,7 +20654,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="1">
+      <c r="D396" s="2">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -20701,7 +20727,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="1">
+      <c r="D398" s="2">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -20739,7 +20765,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="1">
+      <c r="D399" s="2">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -20777,7 +20803,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="1">
+      <c r="D400" s="2">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -20844,7 +20870,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="1">
+      <c r="D402" s="2">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -20917,7 +20943,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="1">
+      <c r="D404" s="2">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -20958,7 +20984,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="1">
+      <c r="D405" s="2">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -20999,7 +21025,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="1">
+      <c r="D406" s="2">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21040,7 +21066,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="1">
+      <c r="D407" s="2">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21107,7 +21133,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="1">
+      <c r="D409" s="2">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21148,7 +21174,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="1">
+      <c r="D410" s="2">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21186,7 +21212,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="1">
+      <c r="D411" s="2">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21224,7 +21250,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="1">
+      <c r="D412" s="2">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21259,7 +21285,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="1">
+      <c r="D413" s="2">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21396,7 +21422,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="1">
+      <c r="D417" s="2">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21431,7 +21457,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="1">
+      <c r="D418" s="2">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21466,7 +21492,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="1">
+      <c r="D419" s="2">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21533,7 +21559,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="1">
+      <c r="D421" s="2">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -21574,7 +21600,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="1">
+      <c r="D422" s="2">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -21615,7 +21641,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="1">
+      <c r="D423" s="2">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -21656,7 +21682,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="1">
+      <c r="D424" s="2">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -21694,7 +21720,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="1">
+      <c r="D425" s="2">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -21735,7 +21761,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="1">
+      <c r="D426" s="2">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -21776,7 +21802,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="1">
+      <c r="D427" s="2">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -21974,7 +22000,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="1">
+      <c r="D433" s="2">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22015,7 +22041,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="1">
+      <c r="D434" s="2">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22146,7 +22172,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="1">
+      <c r="D438" s="2">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22187,7 +22213,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="1">
+      <c r="D439" s="2">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22228,7 +22254,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="1">
+      <c r="D440" s="2">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22269,7 +22295,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="1">
+      <c r="D441" s="2">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22307,7 +22333,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="1">
+      <c r="D442" s="2">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22348,7 +22374,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="1">
+      <c r="D443" s="2">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22389,7 +22415,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="1">
+      <c r="D444" s="2">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22424,7 +22450,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="1">
+      <c r="D445" s="2">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22459,7 +22485,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="1">
+      <c r="D446" s="2">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22526,7 +22552,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="1">
+      <c r="D448" s="2">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22567,7 +22593,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="1">
+      <c r="D449" s="2">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -22602,7 +22628,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="1">
+      <c r="D450" s="2">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -22637,7 +22663,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="1">
+      <c r="D451" s="2">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -22710,7 +22736,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="1">
+      <c r="D453" s="2">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -22751,7 +22777,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="1">
+      <c r="D454" s="2">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -22789,7 +22815,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="1">
+      <c r="D455" s="2">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -22824,7 +22850,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="1">
+      <c r="D456" s="2">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -22923,7 +22949,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="1">
+      <c r="D459" s="2">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -22967,7 +22993,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="1">
+      <c r="D460" s="2">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23034,7 +23060,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="1">
+      <c r="D462" s="2">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23133,7 +23159,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="1">
+      <c r="D465" s="2">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23174,7 +23200,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="1">
+      <c r="D466" s="2">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23215,7 +23241,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="1">
+      <c r="D467" s="2">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23256,7 +23282,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="1">
+      <c r="D468" s="2">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23294,7 +23320,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="1">
+      <c r="D469" s="2">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23332,7 +23358,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="1">
+      <c r="D470" s="2">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23370,7 +23396,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="1">
+      <c r="D471" s="2">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23411,7 +23437,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="1">
+      <c r="D472" s="2">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23449,7 +23475,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="1">
+      <c r="D473" s="2">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23487,7 +23513,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="1">
+      <c r="D474" s="2">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23525,7 +23551,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="1">
+      <c r="D475" s="2">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -23598,7 +23624,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="1">
+      <c r="D477" s="2">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -23770,7 +23796,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="1">
+      <c r="D482" s="2">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -23811,7 +23837,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="1">
+      <c r="D483" s="2">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -23852,7 +23878,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="1">
+      <c r="D484" s="2">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24117,7 +24143,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="1">
+      <c r="D492" s="2">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24158,7 +24184,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="1">
+      <c r="D493" s="2">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24263,7 +24289,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="1">
+      <c r="D496" s="2">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24307,7 +24333,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="1">
+      <c r="D497" s="2">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24348,7 +24374,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="1">
+      <c r="D498" s="2">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24386,7 +24412,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="1">
+      <c r="D499" s="2">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24462,7 +24488,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="1">
+      <c r="D501" s="2">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24506,7 +24532,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="1">
+      <c r="D502" s="2">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24547,7 +24573,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="1">
+      <c r="D503" s="2">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -24652,7 +24678,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="1">
+      <c r="D506" s="2">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -24696,7 +24722,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="1">
+      <c r="D507" s="2">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -24772,7 +24798,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="1">
+      <c r="D509" s="2">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -24807,7 +24833,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="1">
+      <c r="D510" s="2">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -24848,7 +24874,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="1">
+      <c r="D511" s="2">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -24883,7 +24909,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="1">
+      <c r="D512" s="2">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -24924,7 +24950,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="1">
+      <c r="D513" s="2">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -24965,7 +24991,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="1">
+      <c r="D514" s="2">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25006,7 +25032,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="1">
+      <c r="D515" s="2">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25047,7 +25073,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="1">
+      <c r="D516" s="2">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25152,7 +25178,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="1">
+      <c r="D519" s="2">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25286,7 +25312,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="1">
+      <c r="D523" s="2">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25423,7 +25449,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="1">
+      <c r="D527" s="2">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25560,7 +25586,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="1">
+      <c r="D531" s="2">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -25665,7 +25691,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="1">
+      <c r="D534" s="2">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -25703,7 +25729,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="1">
+      <c r="D535" s="2">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -25904,7 +25930,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="1">
+      <c r="D541" s="2">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -25948,7 +25974,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="1">
+      <c r="D542" s="2">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -25983,7 +26009,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="1">
+      <c r="D543" s="2">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26018,7 +26044,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="1">
+      <c r="D544" s="2">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26216,7 +26242,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="1">
+      <c r="D550" s="2">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26321,7 +26347,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="1">
+      <c r="D553" s="2">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26362,7 +26388,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="1">
+      <c r="D554" s="2">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26528,7 +26554,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="1">
+      <c r="D559" s="2">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -26726,7 +26752,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="1">
+      <c r="D565" s="2">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27346,7 +27372,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="1">
+      <c r="D584" s="2">
         <v>46226</v>
       </c>
       <c r="F584" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (06/10/2026 14:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5564,16 +5564,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5589,7 +5581,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5597,30 +5589,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5920,52 +5894,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -6043,7 +6017,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -6180,7 +6154,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -6317,7 +6291,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -6358,7 +6332,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -6393,7 +6367,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6434,7 +6408,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6472,7 +6446,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6513,7 +6487,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6554,7 +6528,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6592,7 +6566,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6633,7 +6607,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6674,7 +6648,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6715,7 +6689,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6756,7 +6730,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6858,7 +6832,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6899,7 +6873,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6940,7 +6914,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6981,7 +6955,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -7022,7 +6996,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -7063,7 +7037,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -7136,7 +7110,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -7209,7 +7183,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -7250,7 +7224,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -7291,7 +7265,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -7332,7 +7306,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7405,7 +7379,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7510,7 +7484,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7551,7 +7525,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7592,7 +7566,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7633,7 +7607,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7674,7 +7648,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7715,7 +7689,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7753,7 +7727,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7794,7 +7768,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7835,7 +7809,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7908,7 +7882,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7949,7 +7923,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -8022,7 +7996,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -8095,7 +8069,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -8168,7 +8142,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -8238,7 +8212,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -8311,7 +8285,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -8346,7 +8320,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -8387,7 +8361,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8428,7 +8402,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8469,7 +8443,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8510,7 +8484,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8551,7 +8525,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8592,7 +8566,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8633,7 +8607,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8668,7 +8642,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8709,7 +8683,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8747,7 +8721,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8785,7 +8759,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8823,7 +8797,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8861,7 +8835,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8902,7 +8876,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8943,7 +8917,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8984,7 +8958,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -9025,7 +8999,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -9066,7 +9040,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -9107,7 +9081,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -9148,7 +9122,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -9189,7 +9163,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -9268,7 +9242,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -9309,7 +9283,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -9350,7 +9324,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -9391,7 +9365,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9432,7 +9406,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9473,7 +9447,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9514,7 +9488,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9555,7 +9529,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9628,7 +9602,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9669,7 +9643,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9710,7 +9684,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9751,7 +9725,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9792,7 +9766,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9830,7 +9804,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9900,7 +9874,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9941,7 +9915,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9982,7 +9956,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -10023,7 +9997,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -10125,7 +10099,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -10166,7 +10140,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -10207,7 +10181,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -10248,7 +10222,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -10286,7 +10260,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -10324,7 +10298,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -10365,7 +10339,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10406,7 +10380,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10447,7 +10421,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10488,7 +10462,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10529,7 +10503,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10570,7 +10544,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10611,7 +10585,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10652,7 +10626,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10690,7 +10664,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10731,7 +10705,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10772,7 +10746,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10842,7 +10816,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10915,7 +10889,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10956,7 +10930,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -10997,7 +10971,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -11070,7 +11044,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -11111,7 +11085,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -11152,7 +11126,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -11190,7 +11164,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -11263,7 +11237,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -11301,7 +11275,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -11371,7 +11345,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11476,7 +11450,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11517,7 +11491,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11558,7 +11532,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11599,7 +11573,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11640,7 +11614,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11681,7 +11655,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11722,7 +11696,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11795,7 +11769,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11836,7 +11810,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11877,7 +11851,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11918,7 +11892,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11988,7 +11962,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -12029,7 +12003,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -12070,7 +12044,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -12111,7 +12085,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -12152,7 +12126,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -12193,7 +12167,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -12231,7 +12205,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -12304,7 +12278,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -12345,7 +12319,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -12383,7 +12357,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12418,7 +12392,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12459,7 +12433,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12500,7 +12474,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12579,7 +12553,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12620,7 +12594,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12661,7 +12635,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12702,7 +12676,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12743,7 +12717,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12784,7 +12758,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12825,7 +12799,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12866,7 +12840,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12939,7 +12913,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -13006,7 +12980,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -13079,7 +13053,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -13120,7 +13094,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -13161,7 +13135,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -13202,7 +13176,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -13243,7 +13217,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -13284,7 +13258,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -13357,7 +13331,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -13398,7 +13372,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13439,7 +13413,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13480,7 +13454,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13521,7 +13495,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13562,7 +13536,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13600,7 +13574,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13641,7 +13615,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13720,7 +13694,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13761,7 +13735,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13802,7 +13776,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13843,7 +13817,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13881,7 +13855,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13922,7 +13896,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13963,7 +13937,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -14001,7 +13975,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -14042,7 +14016,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -14083,7 +14057,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -14124,7 +14098,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -14238,7 +14212,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -14279,7 +14253,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -14320,7 +14294,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -14361,7 +14335,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -14402,7 +14376,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14763,7 +14737,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14804,7 +14778,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14845,7 +14819,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14886,7 +14860,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14927,7 +14901,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14968,7 +14942,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -15009,7 +14983,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -15146,7 +15120,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -15187,7 +15161,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -15260,7 +15234,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -15301,7 +15275,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -15339,7 +15313,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -15377,7 +15351,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15639,7 +15613,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15744,7 +15718,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15785,7 +15759,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15826,7 +15800,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15867,7 +15841,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15905,7 +15879,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15946,7 +15920,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15987,7 +15961,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -16028,7 +16002,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -16072,7 +16046,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -16113,7 +16087,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -16154,7 +16128,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -16195,7 +16169,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -16236,7 +16210,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -16280,7 +16254,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -16315,7 +16289,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -16353,7 +16327,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -16388,7 +16362,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16429,7 +16403,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16467,7 +16441,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16508,7 +16482,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16546,7 +16520,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16584,7 +16558,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16622,7 +16596,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16660,7 +16634,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16701,7 +16675,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16739,7 +16713,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16780,7 +16754,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16821,7 +16795,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16926,7 +16900,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16967,7 +16941,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -17008,7 +16982,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -17049,7 +17023,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -17090,7 +17064,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -17131,7 +17105,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -17172,7 +17146,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -17213,7 +17187,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -17254,7 +17228,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -17289,7 +17263,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -17324,7 +17298,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -17359,7 +17333,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17432,7 +17406,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17473,7 +17447,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17514,7 +17488,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17555,7 +17529,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17593,7 +17567,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17634,7 +17608,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17675,7 +17649,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17716,7 +17690,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17757,7 +17731,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17798,7 +17772,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17839,7 +17813,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17880,7 +17854,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17921,7 +17895,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17956,7 +17930,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -17997,7 +17971,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -18038,7 +18012,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -18079,7 +18053,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -18120,7 +18094,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -18161,7 +18135,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -18202,7 +18176,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -18243,7 +18217,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -18348,7 +18322,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -18389,7 +18363,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18526,7 +18500,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18596,7 +18570,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18637,7 +18611,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18669,7 +18643,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18710,7 +18684,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18748,7 +18722,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18786,7 +18760,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18824,7 +18798,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18859,7 +18833,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18897,7 +18871,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18935,7 +18909,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18973,7 +18947,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -19011,7 +18985,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -19049,7 +19023,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -19087,7 +19061,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -19125,7 +19099,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -19166,7 +19140,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -19271,7 +19245,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -19376,7 +19350,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19414,7 +19388,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19484,7 +19458,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19519,7 +19493,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19557,7 +19531,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19601,7 +19575,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19636,7 +19610,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19674,7 +19648,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19750,7 +19724,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19788,7 +19762,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19858,7 +19832,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19899,7 +19873,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19937,7 +19911,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19975,7 +19949,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -20019,7 +19993,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -20057,7 +20031,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -20098,7 +20072,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -20139,7 +20113,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -20180,7 +20154,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -20346,7 +20320,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -20387,7 +20361,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20428,7 +20402,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20469,7 +20443,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20510,7 +20484,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20551,7 +20525,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20592,7 +20566,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20633,7 +20607,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20674,7 +20648,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20747,7 +20721,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20977,7 +20951,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -21018,7 +20992,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -21059,7 +21033,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -21132,7 +21106,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -21170,7 +21144,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -21208,7 +21182,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -21275,7 +21249,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -21348,7 +21322,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -21389,7 +21363,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21430,7 +21404,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21471,7 +21445,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21538,7 +21512,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21579,7 +21553,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21617,7 +21591,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21655,7 +21629,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21690,7 +21664,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21827,7 +21801,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21862,7 +21836,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21897,7 +21871,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21964,7 +21938,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -22005,7 +21979,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -22046,7 +22020,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -22087,7 +22061,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -22125,7 +22099,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -22166,7 +22140,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -22207,7 +22181,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22405,7 +22379,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22446,7 +22420,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22577,7 +22551,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22618,7 +22592,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22659,7 +22633,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22700,7 +22674,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22738,7 +22712,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22779,7 +22753,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22820,7 +22794,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22855,7 +22829,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22890,7 +22864,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22957,7 +22931,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -22998,7 +22972,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -23033,7 +23007,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -23068,7 +23042,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -23141,7 +23115,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -23182,7 +23156,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -23220,7 +23194,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -23255,7 +23229,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -23354,7 +23328,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -23398,7 +23372,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23465,7 +23439,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23564,7 +23538,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23605,7 +23579,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23646,7 +23620,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23687,7 +23661,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23725,7 +23699,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23763,7 +23737,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23801,7 +23775,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23842,7 +23816,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23880,7 +23854,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23918,7 +23892,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23956,7 +23930,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -24029,7 +24003,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -24201,7 +24175,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -24242,7 +24216,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -24283,7 +24257,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24548,7 +24522,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24589,7 +24563,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24694,7 +24668,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24738,7 +24712,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24779,7 +24753,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24817,7 +24791,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24893,7 +24867,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24937,7 +24911,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24978,7 +24952,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -25083,7 +25057,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -25127,7 +25101,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -25203,7 +25177,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -25238,7 +25212,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -25279,7 +25253,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -25314,7 +25288,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -25355,7 +25329,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -25396,7 +25370,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25437,7 +25411,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25478,7 +25452,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25583,7 +25557,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25717,7 +25691,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25854,7 +25828,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25991,7 +25965,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -26096,7 +26070,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -26134,7 +26108,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -26335,7 +26309,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -26379,7 +26353,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26414,7 +26388,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26449,7 +26423,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26647,7 +26621,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26752,7 +26726,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26793,7 +26767,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26959,7 +26933,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -27157,7 +27131,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27777,7 +27751,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">
@@ -28301,7 +28275,7 @@
       <c r="C600">
         <v>2026</v>
       </c>
-      <c r="D600" s="2">
+      <c r="D600" s="1">
         <v>45802</v>
       </c>
       <c r="F600" t="s">
@@ -28345,7 +28319,7 @@
       <c r="C601">
         <v>2026</v>
       </c>
-      <c r="D601" s="2">
+      <c r="D601" s="1">
         <v>45860</v>
       </c>
       <c r="F601" t="s">
@@ -28386,7 +28360,7 @@
       <c r="C602">
         <v>2026</v>
       </c>
-      <c r="D602" s="2">
+      <c r="D602" s="1">
         <v>45860</v>
       </c>
       <c r="H602" t="s">
@@ -28421,7 +28395,7 @@
       <c r="C603">
         <v>2026</v>
       </c>
-      <c r="D603" s="2">
+      <c r="D603" s="1">
         <v>45856</v>
       </c>
       <c r="F603" t="s">
@@ -28462,7 +28436,7 @@
       <c r="C604">
         <v>2026</v>
       </c>
-      <c r="D604" s="2">
+      <c r="D604" s="1">
         <v>46101</v>
       </c>
       <c r="F604" t="s">
@@ -28503,7 +28477,7 @@
       <c r="C605">
         <v>2026</v>
       </c>
-      <c r="D605" s="2">
+      <c r="D605" s="1">
         <v>46101</v>
       </c>
       <c r="F605" t="s">
@@ -28544,7 +28518,7 @@
       <c r="C606">
         <v>2026</v>
       </c>
-      <c r="D606" s="2">
+      <c r="D606" s="1">
         <v>45863</v>
       </c>
       <c r="F606" t="s">
@@ -28585,7 +28559,7 @@
       <c r="C607">
         <v>2026</v>
       </c>
-      <c r="D607" s="2">
+      <c r="D607" s="1">
         <v>45863</v>
       </c>
       <c r="F607" t="s">
@@ -28626,7 +28600,7 @@
       <c r="C608">
         <v>2026</v>
       </c>
-      <c r="D608" s="2">
+      <c r="D608" s="1">
         <v>46086</v>
       </c>
       <c r="F608" t="s">
@@ -28667,7 +28641,7 @@
       <c r="C609">
         <v>2026</v>
       </c>
-      <c r="D609" s="2">
+      <c r="D609" s="1">
         <v>45874</v>
       </c>
       <c r="F609" t="s">
@@ -28708,7 +28682,7 @@
       <c r="C610">
         <v>2026</v>
       </c>
-      <c r="D610" s="2">
+      <c r="D610" s="1">
         <v>45894</v>
       </c>
       <c r="F610" t="s">
@@ -28749,7 +28723,7 @@
       <c r="C611">
         <v>2026</v>
       </c>
-      <c r="D611" s="2">
+      <c r="D611" s="1">
         <v>45894</v>
       </c>
       <c r="F611" t="s">
@@ -28790,7 +28764,7 @@
       <c r="C612">
         <v>2026</v>
       </c>
-      <c r="D612" s="2">
+      <c r="D612" s="1">
         <v>46119</v>
       </c>
       <c r="F612" t="s">
@@ -28831,7 +28805,7 @@
       <c r="C613">
         <v>2026</v>
       </c>
-      <c r="D613" s="2">
+      <c r="D613" s="1">
         <v>45898</v>
       </c>
       <c r="F613" t="s">
@@ -28872,7 +28846,7 @@
       <c r="C614">
         <v>2026</v>
       </c>
-      <c r="D614" s="2">
+      <c r="D614" s="1">
         <v>45971</v>
       </c>
       <c r="F614" t="s">
@@ -28913,7 +28887,7 @@
       <c r="C615">
         <v>2026</v>
       </c>
-      <c r="D615" s="2">
+      <c r="D615" s="1">
         <v>46119</v>
       </c>
       <c r="F615" t="s">
@@ -28954,7 +28928,7 @@
       <c r="C616">
         <v>2026</v>
       </c>
-      <c r="D616" s="2">
+      <c r="D616" s="1">
         <v>46092</v>
       </c>
       <c r="F616" t="s">
@@ -28995,7 +28969,7 @@
       <c r="C617">
         <v>2026</v>
       </c>
-      <c r="D617" s="2">
+      <c r="D617" s="1">
         <v>46119</v>
       </c>
       <c r="F617" t="s">
@@ -29036,7 +29010,7 @@
       <c r="C618">
         <v>2026</v>
       </c>
-      <c r="D618" s="2">
+      <c r="D618" s="1">
         <v>46029</v>
       </c>
       <c r="F618" t="s">
@@ -29077,7 +29051,7 @@
       <c r="C619">
         <v>2026</v>
       </c>
-      <c r="D619" s="2">
+      <c r="D619" s="1">
         <v>46029</v>
       </c>
       <c r="F619" t="s">
@@ -29118,7 +29092,7 @@
       <c r="C620">
         <v>2026</v>
       </c>
-      <c r="D620" s="2">
+      <c r="D620" s="1">
         <v>46063</v>
       </c>
       <c r="H620" t="s">
@@ -29153,7 +29127,7 @@
       <c r="C621">
         <v>2026</v>
       </c>
-      <c r="D621" s="2">
+      <c r="D621" s="1">
         <v>46232</v>
       </c>
       <c r="G621" t="s">
@@ -29191,7 +29165,7 @@
       <c r="C622">
         <v>2026</v>
       </c>
-      <c r="D622" s="2">
+      <c r="D622" s="1">
         <v>46232</v>
       </c>
       <c r="G622" t="s">
@@ -29229,7 +29203,7 @@
       <c r="C623">
         <v>2026</v>
       </c>
-      <c r="D623" s="2">
+      <c r="D623" s="1">
         <v>46232</v>
       </c>
       <c r="G623" t="s">
@@ -29267,7 +29241,7 @@
       <c r="C624">
         <v>2026</v>
       </c>
-      <c r="D624" s="2">
+      <c r="D624" s="1">
         <v>46232</v>
       </c>
       <c r="G624" t="s">
@@ -29305,7 +29279,7 @@
       <c r="C625">
         <v>2026</v>
       </c>
-      <c r="D625" s="2">
+      <c r="D625" s="1">
         <v>46155</v>
       </c>
       <c r="H625" t="s">
@@ -29340,7 +29314,7 @@
       <c r="C626">
         <v>2026</v>
       </c>
-      <c r="D626" s="2">
+      <c r="D626" s="1">
         <v>46139</v>
       </c>
       <c r="F626" t="s">
@@ -29381,7 +29355,7 @@
       <c r="C627">
         <v>2026</v>
       </c>
-      <c r="D627" s="2">
+      <c r="D627" s="1">
         <v>46155</v>
       </c>
       <c r="F627" t="s">
@@ -29422,7 +29396,7 @@
       <c r="C628">
         <v>2026</v>
       </c>
-      <c r="D628" s="2">
+      <c r="D628" s="1">
         <v>46155</v>
       </c>
       <c r="H628" t="s">
@@ -29457,7 +29431,7 @@
       <c r="C629">
         <v>2026</v>
       </c>
-      <c r="D629" s="2">
+      <c r="D629" s="1">
         <v>46147</v>
       </c>
       <c r="H629" t="s">
@@ -29492,7 +29466,7 @@
       <c r="C630">
         <v>2026</v>
       </c>
-      <c r="D630" s="2">
+      <c r="D630" s="1">
         <v>46164</v>
       </c>
       <c r="F630" t="s">
@@ -29533,7 +29507,7 @@
       <c r="C631">
         <v>2026</v>
       </c>
-      <c r="D631" s="2">
+      <c r="D631" s="1">
         <v>46225</v>
       </c>
       <c r="F631" t="s">
@@ -29574,7 +29548,7 @@
       <c r="C632">
         <v>2026</v>
       </c>
-      <c r="D632" s="2">
+      <c r="D632" s="1">
         <v>46225</v>
       </c>
       <c r="F632" t="s">
@@ -29615,7 +29589,7 @@
       <c r="C633">
         <v>2026</v>
       </c>
-      <c r="D633" s="2">
+      <c r="D633" s="1">
         <v>46225</v>
       </c>
       <c r="F633" t="s">
@@ -29656,7 +29630,7 @@
       <c r="C634">
         <v>2026</v>
       </c>
-      <c r="D634" s="2">
+      <c r="D634" s="1">
         <v>46248</v>
       </c>
       <c r="H634" t="s">
@@ -29691,7 +29665,7 @@
       <c r="C635">
         <v>2026</v>
       </c>
-      <c r="D635" s="2">
+      <c r="D635" s="1">
         <v>46248</v>
       </c>
       <c r="F635" t="s">
@@ -29732,7 +29706,7 @@
       <c r="C636">
         <v>2026</v>
       </c>
-      <c r="D636" s="2">
+      <c r="D636" s="1">
         <v>46171</v>
       </c>
       <c r="H636" t="s">
@@ -29767,7 +29741,7 @@
       <c r="C637">
         <v>2026</v>
       </c>
-      <c r="D637" s="2">
+      <c r="D637" s="1">
         <v>46176</v>
       </c>
       <c r="H637" t="s">
@@ -29802,7 +29776,7 @@
       <c r="C638">
         <v>2026</v>
       </c>
-      <c r="D638" s="2">
+      <c r="D638" s="1">
         <v>46225</v>
       </c>
       <c r="F638" t="s">
@@ -29843,7 +29817,7 @@
       <c r="C639">
         <v>2026</v>
       </c>
-      <c r="D639" s="2">
+      <c r="D639" s="1">
         <v>46211</v>
       </c>
       <c r="H639" t="s">
@@ -29878,7 +29852,7 @@
       <c r="C640">
         <v>2026</v>
       </c>
-      <c r="D640" s="2">
+      <c r="D640" s="1">
         <v>46183</v>
       </c>
       <c r="H640" t="s">
@@ -29913,7 +29887,7 @@
       <c r="C641">
         <v>2026</v>
       </c>
-      <c r="D641" s="2">
+      <c r="D641" s="1">
         <v>46191</v>
       </c>
       <c r="F641" t="s">
@@ -29954,7 +29928,7 @@
       <c r="C642">
         <v>2026</v>
       </c>
-      <c r="D642" s="2">
+      <c r="D642" s="1">
         <v>46176</v>
       </c>
       <c r="H642" t="s">
@@ -29989,7 +29963,7 @@
       <c r="C643">
         <v>2026</v>
       </c>
-      <c r="D643" s="2">
+      <c r="D643" s="1">
         <v>46191</v>
       </c>
       <c r="H643" t="s">
@@ -30024,7 +29998,7 @@
       <c r="C644">
         <v>2026</v>
       </c>
-      <c r="D644" s="2">
+      <c r="D644" s="1">
         <v>46241</v>
       </c>
       <c r="F644" t="s">
@@ -30068,7 +30042,7 @@
       <c r="C645">
         <v>2026</v>
       </c>
-      <c r="D645" s="2">
+      <c r="D645" s="1">
         <v>46191</v>
       </c>
       <c r="F645" t="s">
@@ -30109,7 +30083,7 @@
       <c r="C646">
         <v>2026</v>
       </c>
-      <c r="D646" s="2">
+      <c r="D646" s="1">
         <v>46191</v>
       </c>
       <c r="F646" t="s">
@@ -30150,7 +30124,7 @@
       <c r="C647">
         <v>2026</v>
       </c>
-      <c r="D647" s="2">
+      <c r="D647" s="1">
         <v>46191</v>
       </c>
       <c r="H647" t="s">
@@ -30185,7 +30159,7 @@
       <c r="C648">
         <v>2026</v>
       </c>
-      <c r="D648" s="2">
+      <c r="D648" s="1">
         <v>46241</v>
       </c>
       <c r="F648" t="s">
@@ -30226,7 +30200,7 @@
       <c r="C649">
         <v>2026</v>
       </c>
-      <c r="D649" s="2">
+      <c r="D649" s="1">
         <v>46191</v>
       </c>
       <c r="H649" t="s">
@@ -30261,7 +30235,7 @@
       <c r="C650">
         <v>2026</v>
       </c>
-      <c r="D650" s="2">
+      <c r="D650" s="1">
         <v>46248</v>
       </c>
       <c r="H650" t="s">
@@ -30296,7 +30270,7 @@
       <c r="C651">
         <v>2026</v>
       </c>
-      <c r="D651" s="2">
+      <c r="D651" s="1">
         <v>46241</v>
       </c>
       <c r="F651" t="s">
@@ -30337,7 +30311,7 @@
       <c r="C652">
         <v>2026</v>
       </c>
-      <c r="D652" s="2">
+      <c r="D652" s="1">
         <v>46241</v>
       </c>
       <c r="F652" t="s">
@@ -30378,7 +30352,7 @@
       <c r="C653">
         <v>2026</v>
       </c>
-      <c r="D653" s="2">
+      <c r="D653" s="1">
         <v>46225</v>
       </c>
       <c r="F653" t="s">
@@ -30419,7 +30393,7 @@
       <c r="C654">
         <v>2026</v>
       </c>
-      <c r="D654" s="2">
+      <c r="D654" s="1">
         <v>46241</v>
       </c>
       <c r="F654" t="s">
@@ -30460,7 +30434,7 @@
       <c r="C655">
         <v>2026</v>
       </c>
-      <c r="D655" s="2">
+      <c r="D655" s="1">
         <v>46241</v>
       </c>
       <c r="F655" t="s">
@@ -30501,7 +30475,7 @@
       <c r="C656">
         <v>2026</v>
       </c>
-      <c r="D656" s="2">
+      <c r="D656" s="1">
         <v>46241</v>
       </c>
       <c r="F656" t="s">
@@ -30542,7 +30516,7 @@
       <c r="C657">
         <v>2026</v>
       </c>
-      <c r="D657" s="2">
+      <c r="D657" s="1">
         <v>46248</v>
       </c>
       <c r="H657" t="s">
@@ -30577,7 +30551,7 @@
       <c r="C658">
         <v>2026</v>
       </c>
-      <c r="D658" s="2">
+      <c r="D658" s="1">
         <v>46248</v>
       </c>
       <c r="H658" t="s">
@@ -30612,7 +30586,7 @@
       <c r="C659">
         <v>2026</v>
       </c>
-      <c r="D659" s="2">
+      <c r="D659" s="1">
         <v>46248</v>
       </c>
       <c r="F659" t="s">
@@ -30653,7 +30627,7 @@
       <c r="C660">
         <v>2026</v>
       </c>
-      <c r="D660" s="2">
+      <c r="D660" s="1">
         <v>46248</v>
       </c>
       <c r="F660" t="s">
@@ -30694,7 +30668,7 @@
       <c r="C661">
         <v>2026</v>
       </c>
-      <c r="D661" s="2">
+      <c r="D661" s="1">
         <v>46248</v>
       </c>
       <c r="F661" t="s">
@@ -30735,7 +30709,7 @@
       <c r="C662">
         <v>2026</v>
       </c>
-      <c r="D662" s="2">
+      <c r="D662" s="1">
         <v>45989</v>
       </c>
       <c r="G662" t="s">
@@ -30773,7 +30747,7 @@
       <c r="C663">
         <v>2026</v>
       </c>
-      <c r="D663" s="2">
+      <c r="D663" s="1">
         <v>46002</v>
       </c>
       <c r="G663" t="s">
@@ -30811,7 +30785,7 @@
       <c r="C664">
         <v>2026</v>
       </c>
-      <c r="D664" s="2">
+      <c r="D664" s="1">
         <v>46002</v>
       </c>
       <c r="G664" t="s">
@@ -30849,7 +30823,7 @@
       <c r="C665">
         <v>2026</v>
       </c>
-      <c r="D665" s="2">
+      <c r="D665" s="1">
         <v>46225</v>
       </c>
       <c r="F665" t="s">
@@ -30890,7 +30864,7 @@
       <c r="C666">
         <v>2026</v>
       </c>
-      <c r="D666" s="2">
+      <c r="D666" s="1">
         <v>46211</v>
       </c>
       <c r="F666" t="s">
@@ -30931,7 +30905,7 @@
       <c r="C667">
         <v>2026</v>
       </c>
-      <c r="D667" s="2">
+      <c r="D667" s="1">
         <v>46248</v>
       </c>
       <c r="F667" t="s">
@@ -30972,7 +30946,7 @@
       <c r="C668">
         <v>2026</v>
       </c>
-      <c r="D668" s="2">
+      <c r="D668" s="1">
         <v>46248</v>
       </c>
       <c r="F668" t="s">
@@ -31045,7 +31019,7 @@
       <c r="C670">
         <v>2026</v>
       </c>
-      <c r="D670" s="2">
+      <c r="D670" s="1">
         <v>46255</v>
       </c>
       <c r="F670" t="s">
@@ -31246,7 +31220,7 @@
       <c r="C676">
         <v>2026</v>
       </c>
-      <c r="D676" s="2">
+      <c r="D676" s="1">
         <v>46265</v>
       </c>
       <c r="H676" t="s">
@@ -31281,7 +31255,7 @@
       <c r="C677">
         <v>2026</v>
       </c>
-      <c r="D677" s="2">
+      <c r="D677" s="1">
         <v>46265</v>
       </c>
       <c r="H677" t="s">
@@ -31316,7 +31290,7 @@
       <c r="C678">
         <v>2026</v>
       </c>
-      <c r="D678" s="2">
+      <c r="D678" s="1">
         <v>46265</v>
       </c>
       <c r="H678" t="s">
@@ -31671,7 +31645,7 @@
       <c r="C689">
         <v>2026</v>
       </c>
-      <c r="D689" s="2">
+      <c r="D689" s="1">
         <v>46265</v>
       </c>
       <c r="H689" t="s">
@@ -31706,7 +31680,7 @@
       <c r="C690">
         <v>2026</v>
       </c>
-      <c r="D690" s="2">
+      <c r="D690" s="1">
         <v>46265</v>
       </c>
       <c r="H690" t="s">

</xml_diff>

<commit_message>
Atualização automática: reparaveis_rma (07/10/2026 14:48)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/reparaveis_complemento_rma.xlsx
@@ -5570,16 +5570,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5595,7 +5587,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5603,30 +5595,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5926,52 +5900,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -6049,7 +6023,7 @@
       <c r="C4">
         <v>2026</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45972</v>
       </c>
       <c r="F4" t="s">
@@ -6186,7 +6160,7 @@
       <c r="C8">
         <v>2026</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>46014</v>
       </c>
       <c r="F8" t="s">
@@ -6323,7 +6297,7 @@
       <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45916</v>
       </c>
       <c r="F12" t="s">
@@ -6364,7 +6338,7 @@
       <c r="C13">
         <v>2026</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45897</v>
       </c>
       <c r="H13" t="s">
@@ -6399,7 +6373,7 @@
       <c r="C14">
         <v>2026</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45916</v>
       </c>
       <c r="F14" t="s">
@@ -6440,7 +6414,7 @@
       <c r="C15">
         <v>2026</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46086</v>
       </c>
       <c r="G15" t="s">
@@ -6478,7 +6452,7 @@
       <c r="C16">
         <v>2026</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45869</v>
       </c>
       <c r="F16" t="s">
@@ -6519,7 +6493,7 @@
       <c r="C17">
         <v>2026</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45877</v>
       </c>
       <c r="F17" t="s">
@@ -6560,7 +6534,7 @@
       <c r="C18">
         <v>2026</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>46086</v>
       </c>
       <c r="G18" t="s">
@@ -6598,7 +6572,7 @@
       <c r="C19">
         <v>2026</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45863</v>
       </c>
       <c r="F19" t="s">
@@ -6639,7 +6613,7 @@
       <c r="C20">
         <v>2026</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45863</v>
       </c>
       <c r="F20" t="s">
@@ -6680,7 +6654,7 @@
       <c r="C21">
         <v>2026</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45873</v>
       </c>
       <c r="F21" t="s">
@@ -6721,7 +6695,7 @@
       <c r="C22">
         <v>2026</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>46086</v>
       </c>
       <c r="F22" t="s">
@@ -6762,7 +6736,7 @@
       <c r="C23">
         <v>2026</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>46086</v>
       </c>
       <c r="G23" t="s">
@@ -6864,7 +6838,7 @@
       <c r="C26">
         <v>2026</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>45838</v>
       </c>
       <c r="F26" t="s">
@@ -6905,7 +6879,7 @@
       <c r="C27">
         <v>2026</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="1">
         <v>45800</v>
       </c>
       <c r="F27" t="s">
@@ -6946,7 +6920,7 @@
       <c r="C28">
         <v>2026</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28" s="1">
         <v>45849</v>
       </c>
       <c r="F28" t="s">
@@ -6987,7 +6961,7 @@
       <c r="C29">
         <v>2026</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29" s="1">
         <v>45838</v>
       </c>
       <c r="F29" t="s">
@@ -7028,7 +7002,7 @@
       <c r="C30">
         <v>2026</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30" s="1">
         <v>45915</v>
       </c>
       <c r="F30" t="s">
@@ -7069,7 +7043,7 @@
       <c r="C31">
         <v>2026</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31" s="1">
         <v>45849</v>
       </c>
       <c r="F31" t="s">
@@ -7142,7 +7116,7 @@
       <c r="C33">
         <v>2026</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33" s="1">
         <v>45800</v>
       </c>
       <c r="F33" t="s">
@@ -7215,7 +7189,7 @@
       <c r="C35">
         <v>2026</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <v>46119</v>
       </c>
       <c r="F35" t="s">
@@ -7256,7 +7230,7 @@
       <c r="C36">
         <v>2026</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36" s="1">
         <v>45854</v>
       </c>
       <c r="F36" t="s">
@@ -7297,7 +7271,7 @@
       <c r="C37">
         <v>2026</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37" s="1">
         <v>45849</v>
       </c>
       <c r="F37" t="s">
@@ -7338,7 +7312,7 @@
       <c r="C38">
         <v>2026</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38" s="1">
         <v>46119</v>
       </c>
       <c r="F38" t="s">
@@ -7411,7 +7385,7 @@
       <c r="C40">
         <v>2026</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40" s="1">
         <v>46092</v>
       </c>
       <c r="F40" t="s">
@@ -7516,7 +7490,7 @@
       <c r="C43">
         <v>2026</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43" s="1">
         <v>46122</v>
       </c>
       <c r="F43" t="s">
@@ -7557,7 +7531,7 @@
       <c r="C44">
         <v>2026</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44" s="1">
         <v>46122</v>
       </c>
       <c r="F44" t="s">
@@ -7598,7 +7572,7 @@
       <c r="C45">
         <v>2026</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45" s="1">
         <v>46135</v>
       </c>
       <c r="F45" t="s">
@@ -7639,7 +7613,7 @@
       <c r="C46">
         <v>2026</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46" s="1">
         <v>46086</v>
       </c>
       <c r="F46" t="s">
@@ -7680,7 +7654,7 @@
       <c r="C47">
         <v>2026</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47" s="1">
         <v>46104</v>
       </c>
       <c r="F47" t="s">
@@ -7721,7 +7695,7 @@
       <c r="C48">
         <v>2026</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48" s="1">
         <v>45972</v>
       </c>
       <c r="G48" t="s">
@@ -7759,7 +7733,7 @@
       <c r="C49">
         <v>2026</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49" s="1">
         <v>45810</v>
       </c>
       <c r="F49" t="s">
@@ -7800,7 +7774,7 @@
       <c r="C50">
         <v>2026</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50" s="1">
         <v>45937</v>
       </c>
       <c r="F50" t="s">
@@ -7841,7 +7815,7 @@
       <c r="C51">
         <v>2026</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51" s="1">
         <v>45937</v>
       </c>
       <c r="F51" t="s">
@@ -7914,7 +7888,7 @@
       <c r="C53">
         <v>2026</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53" s="1">
         <v>45845</v>
       </c>
       <c r="F53" t="s">
@@ -7955,7 +7929,7 @@
       <c r="C54">
         <v>2026</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54" s="1">
         <v>46077</v>
       </c>
       <c r="F54" t="s">
@@ -8028,7 +8002,7 @@
       <c r="C56">
         <v>2026</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56" s="1">
         <v>45971</v>
       </c>
       <c r="F56" t="s">
@@ -8101,7 +8075,7 @@
       <c r="C58">
         <v>2026</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58" s="1">
         <v>45817</v>
       </c>
       <c r="F58" t="s">
@@ -8174,7 +8148,7 @@
       <c r="C60">
         <v>2026</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60" s="1">
         <v>45965</v>
       </c>
       <c r="G60" t="s">
@@ -8244,7 +8218,7 @@
       <c r="C62">
         <v>2026</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62" s="1">
         <v>46072</v>
       </c>
       <c r="F62" t="s">
@@ -8317,7 +8291,7 @@
       <c r="C64">
         <v>2026</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64" s="1">
         <v>46072</v>
       </c>
       <c r="H64" t="s">
@@ -8352,7 +8326,7 @@
       <c r="C65">
         <v>2026</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65" s="1">
         <v>45804</v>
       </c>
       <c r="F65" t="s">
@@ -8393,7 +8367,7 @@
       <c r="C66">
         <v>2026</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66" s="1">
         <v>45804</v>
       </c>
       <c r="F66" t="s">
@@ -8434,7 +8408,7 @@
       <c r="C67">
         <v>2026</v>
       </c>
-      <c r="D67" s="2">
+      <c r="D67" s="1">
         <v>45804</v>
       </c>
       <c r="F67" t="s">
@@ -8475,7 +8449,7 @@
       <c r="C68">
         <v>2026</v>
       </c>
-      <c r="D68" s="2">
+      <c r="D68" s="1">
         <v>45804</v>
       </c>
       <c r="F68" t="s">
@@ -8516,7 +8490,7 @@
       <c r="C69">
         <v>2026</v>
       </c>
-      <c r="D69" s="2">
+      <c r="D69" s="1">
         <v>45804</v>
       </c>
       <c r="F69" t="s">
@@ -8557,7 +8531,7 @@
       <c r="C70">
         <v>2026</v>
       </c>
-      <c r="D70" s="2">
+      <c r="D70" s="1">
         <v>45804</v>
       </c>
       <c r="F70" t="s">
@@ -8598,7 +8572,7 @@
       <c r="C71">
         <v>2026</v>
       </c>
-      <c r="D71" s="2">
+      <c r="D71" s="1">
         <v>45821</v>
       </c>
       <c r="F71" t="s">
@@ -8639,7 +8613,7 @@
       <c r="C72">
         <v>2026</v>
       </c>
-      <c r="D72" s="2">
+      <c r="D72" s="1">
         <v>45821</v>
       </c>
       <c r="H72" t="s">
@@ -8674,7 +8648,7 @@
       <c r="C73">
         <v>2026</v>
       </c>
-      <c r="D73" s="2">
+      <c r="D73" s="1">
         <v>45891</v>
       </c>
       <c r="F73" t="s">
@@ -8715,7 +8689,7 @@
       <c r="C74">
         <v>2026</v>
       </c>
-      <c r="D74" s="2">
+      <c r="D74" s="1">
         <v>45817</v>
       </c>
       <c r="G74" t="s">
@@ -8753,7 +8727,7 @@
       <c r="C75">
         <v>2026</v>
       </c>
-      <c r="D75" s="2">
+      <c r="D75" s="1">
         <v>45883</v>
       </c>
       <c r="G75" t="s">
@@ -8791,7 +8765,7 @@
       <c r="C76">
         <v>2026</v>
       </c>
-      <c r="D76" s="2">
+      <c r="D76" s="1">
         <v>45817</v>
       </c>
       <c r="G76" t="s">
@@ -8829,7 +8803,7 @@
       <c r="C77">
         <v>2026</v>
       </c>
-      <c r="D77" s="2">
+      <c r="D77" s="1">
         <v>45883</v>
       </c>
       <c r="G77" t="s">
@@ -8867,7 +8841,7 @@
       <c r="C78">
         <v>2026</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="1">
         <v>45971</v>
       </c>
       <c r="F78" t="s">
@@ -8908,7 +8882,7 @@
       <c r="C79">
         <v>2026</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D79" s="1">
         <v>45849</v>
       </c>
       <c r="F79" t="s">
@@ -8949,7 +8923,7 @@
       <c r="C80">
         <v>2026</v>
       </c>
-      <c r="D80" s="2">
+      <c r="D80" s="1">
         <v>45849</v>
       </c>
       <c r="F80" t="s">
@@ -8990,7 +8964,7 @@
       <c r="C81">
         <v>2026</v>
       </c>
-      <c r="D81" s="2">
+      <c r="D81" s="1">
         <v>45863</v>
       </c>
       <c r="F81" t="s">
@@ -9031,7 +9005,7 @@
       <c r="C82">
         <v>2026</v>
       </c>
-      <c r="D82" s="2">
+      <c r="D82" s="1">
         <v>45810</v>
       </c>
       <c r="F82" t="s">
@@ -9072,7 +9046,7 @@
       <c r="C83">
         <v>2026</v>
       </c>
-      <c r="D83" s="2">
+      <c r="D83" s="1">
         <v>45926</v>
       </c>
       <c r="F83" t="s">
@@ -9113,7 +9087,7 @@
       <c r="C84">
         <v>2026</v>
       </c>
-      <c r="D84" s="2">
+      <c r="D84" s="1">
         <v>45971</v>
       </c>
       <c r="F84" t="s">
@@ -9154,7 +9128,7 @@
       <c r="C85">
         <v>2026</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="1">
         <v>46164</v>
       </c>
       <c r="F85" t="s">
@@ -9195,7 +9169,7 @@
       <c r="C86">
         <v>2026</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="1">
         <v>45986</v>
       </c>
       <c r="G86" t="s">
@@ -9274,7 +9248,7 @@
       <c r="C88">
         <v>2026</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="1">
         <v>45786</v>
       </c>
       <c r="F88" t="s">
@@ -9315,7 +9289,7 @@
       <c r="C89">
         <v>2026</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="1">
         <v>45777</v>
       </c>
       <c r="F89" t="s">
@@ -9356,7 +9330,7 @@
       <c r="C90">
         <v>2026</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="1">
         <v>45869</v>
       </c>
       <c r="F90" t="s">
@@ -9397,7 +9371,7 @@
       <c r="C91">
         <v>2026</v>
       </c>
-      <c r="D91" s="2">
+      <c r="D91" s="1">
         <v>45891</v>
       </c>
       <c r="F91" t="s">
@@ -9438,7 +9412,7 @@
       <c r="C92">
         <v>2026</v>
       </c>
-      <c r="D92" s="2">
+      <c r="D92" s="1">
         <v>45863</v>
       </c>
       <c r="F92" t="s">
@@ -9479,7 +9453,7 @@
       <c r="C93">
         <v>2026</v>
       </c>
-      <c r="D93" s="2">
+      <c r="D93" s="1">
         <v>45769</v>
       </c>
       <c r="F93" t="s">
@@ -9520,7 +9494,7 @@
       <c r="C94">
         <v>2026</v>
       </c>
-      <c r="D94" s="2">
+      <c r="D94" s="1">
         <v>45769</v>
       </c>
       <c r="F94" t="s">
@@ -9561,7 +9535,7 @@
       <c r="C95">
         <v>2026</v>
       </c>
-      <c r="D95" s="2">
+      <c r="D95" s="1">
         <v>45894</v>
       </c>
       <c r="F95" t="s">
@@ -9634,7 +9608,7 @@
       <c r="C97">
         <v>2026</v>
       </c>
-      <c r="D97" s="2">
+      <c r="D97" s="1">
         <v>45894</v>
       </c>
       <c r="F97" t="s">
@@ -9675,7 +9649,7 @@
       <c r="C98">
         <v>2026</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D98" s="1">
         <v>45971</v>
       </c>
       <c r="F98" t="s">
@@ -9716,7 +9690,7 @@
       <c r="C99">
         <v>2026</v>
       </c>
-      <c r="D99" s="2">
+      <c r="D99" s="1">
         <v>45971</v>
       </c>
       <c r="F99" t="s">
@@ -9757,7 +9731,7 @@
       <c r="C100">
         <v>2026</v>
       </c>
-      <c r="D100" s="2">
+      <c r="D100" s="1">
         <v>45971</v>
       </c>
       <c r="F100" t="s">
@@ -9798,7 +9772,7 @@
       <c r="C101">
         <v>2026</v>
       </c>
-      <c r="D101" s="2">
+      <c r="D101" s="1">
         <v>45996</v>
       </c>
       <c r="G101" t="s">
@@ -9836,7 +9810,7 @@
       <c r="C102">
         <v>2026</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="1">
         <v>45986</v>
       </c>
       <c r="G102" t="s">
@@ -9906,7 +9880,7 @@
       <c r="C104">
         <v>2026</v>
       </c>
-      <c r="D104" s="2">
+      <c r="D104" s="1">
         <v>45769</v>
       </c>
       <c r="F104" t="s">
@@ -9947,7 +9921,7 @@
       <c r="C105">
         <v>2026</v>
       </c>
-      <c r="D105" s="2">
+      <c r="D105" s="1">
         <v>45769</v>
       </c>
       <c r="F105" t="s">
@@ -9988,7 +9962,7 @@
       <c r="C106">
         <v>2026</v>
       </c>
-      <c r="D106" s="2">
+      <c r="D106" s="1">
         <v>45849</v>
       </c>
       <c r="F106" t="s">
@@ -10029,7 +10003,7 @@
       <c r="C107">
         <v>2026</v>
       </c>
-      <c r="D107" s="2">
+      <c r="D107" s="1">
         <v>45849</v>
       </c>
       <c r="G107" t="s">
@@ -10131,7 +10105,7 @@
       <c r="C110">
         <v>2026</v>
       </c>
-      <c r="D110" s="2">
+      <c r="D110" s="1">
         <v>45891</v>
       </c>
       <c r="F110" t="s">
@@ -10172,7 +10146,7 @@
       <c r="C111">
         <v>2026</v>
       </c>
-      <c r="D111" s="2">
+      <c r="D111" s="1">
         <v>45769</v>
       </c>
       <c r="F111" t="s">
@@ -10213,7 +10187,7 @@
       <c r="C112">
         <v>2026</v>
       </c>
-      <c r="D112" s="2">
+      <c r="D112" s="1">
         <v>45889</v>
       </c>
       <c r="F112" t="s">
@@ -10254,7 +10228,7 @@
       <c r="C113">
         <v>2026</v>
       </c>
-      <c r="D113" s="2">
+      <c r="D113" s="1">
         <v>45945</v>
       </c>
       <c r="G113" t="s">
@@ -10292,7 +10266,7 @@
       <c r="C114">
         <v>2026</v>
       </c>
-      <c r="D114" s="2">
+      <c r="D114" s="1">
         <v>45945</v>
       </c>
       <c r="G114" t="s">
@@ -10330,7 +10304,7 @@
       <c r="C115">
         <v>2026</v>
       </c>
-      <c r="D115" s="2">
+      <c r="D115" s="1">
         <v>46119</v>
       </c>
       <c r="F115" t="s">
@@ -10371,7 +10345,7 @@
       <c r="C116">
         <v>2026</v>
       </c>
-      <c r="D116" s="2">
+      <c r="D116" s="1">
         <v>46029</v>
       </c>
       <c r="F116" t="s">
@@ -10412,7 +10386,7 @@
       <c r="C117">
         <v>2026</v>
       </c>
-      <c r="D117" s="2">
+      <c r="D117" s="1">
         <v>46029</v>
       </c>
       <c r="F117" t="s">
@@ -10453,7 +10427,7 @@
       <c r="C118">
         <v>2026</v>
       </c>
-      <c r="D118" s="2">
+      <c r="D118" s="1">
         <v>46119</v>
       </c>
       <c r="F118" t="s">
@@ -10494,7 +10468,7 @@
       <c r="C119">
         <v>2026</v>
       </c>
-      <c r="D119" s="2">
+      <c r="D119" s="1">
         <v>46230</v>
       </c>
       <c r="F119" t="s">
@@ -10535,7 +10509,7 @@
       <c r="C120">
         <v>2026</v>
       </c>
-      <c r="D120" s="2">
+      <c r="D120" s="1">
         <v>46119</v>
       </c>
       <c r="F120" t="s">
@@ -10576,7 +10550,7 @@
       <c r="C121">
         <v>2026</v>
       </c>
-      <c r="D121" s="2">
+      <c r="D121" s="1">
         <v>46119</v>
       </c>
       <c r="F121" t="s">
@@ -10617,7 +10591,7 @@
       <c r="C122">
         <v>2026</v>
       </c>
-      <c r="D122" s="2">
+      <c r="D122" s="1">
         <v>45931</v>
       </c>
       <c r="F122" t="s">
@@ -10658,7 +10632,7 @@
       <c r="C123">
         <v>2026</v>
       </c>
-      <c r="D123" s="2">
+      <c r="D123" s="1">
         <v>45894</v>
       </c>
       <c r="G123" t="s">
@@ -10696,7 +10670,7 @@
       <c r="C124">
         <v>2026</v>
       </c>
-      <c r="D124" s="2">
+      <c r="D124" s="1">
         <v>46119</v>
       </c>
       <c r="F124" t="s">
@@ -10737,7 +10711,7 @@
       <c r="C125">
         <v>2026</v>
       </c>
-      <c r="D125" s="2">
+      <c r="D125" s="1">
         <v>45889</v>
       </c>
       <c r="F125" t="s">
@@ -10778,7 +10752,7 @@
       <c r="C126">
         <v>2026</v>
       </c>
-      <c r="D126" s="2">
+      <c r="D126" s="1">
         <v>45876</v>
       </c>
       <c r="G126" t="s">
@@ -10848,7 +10822,7 @@
       <c r="C128">
         <v>2026</v>
       </c>
-      <c r="D128" s="2">
+      <c r="D128" s="1">
         <v>45876</v>
       </c>
       <c r="F128" t="s">
@@ -10921,7 +10895,7 @@
       <c r="C130">
         <v>2026</v>
       </c>
-      <c r="D130" s="2">
+      <c r="D130" s="1">
         <v>46230</v>
       </c>
       <c r="F130" t="s">
@@ -10962,7 +10936,7 @@
       <c r="C131">
         <v>2026</v>
       </c>
-      <c r="D131" s="2">
+      <c r="D131" s="1">
         <v>45889</v>
       </c>
       <c r="F131" t="s">
@@ -11003,7 +10977,7 @@
       <c r="C132">
         <v>2026</v>
       </c>
-      <c r="D132" s="2">
+      <c r="D132" s="1">
         <v>46230</v>
       </c>
       <c r="F132" t="s">
@@ -11076,7 +11050,7 @@
       <c r="C134">
         <v>2026</v>
       </c>
-      <c r="D134" s="2">
+      <c r="D134" s="1">
         <v>46140</v>
       </c>
       <c r="F134" t="s">
@@ -11117,7 +11091,7 @@
       <c r="C135">
         <v>2026</v>
       </c>
-      <c r="D135" s="2">
+      <c r="D135" s="1">
         <v>45889</v>
       </c>
       <c r="F135" t="s">
@@ -11158,7 +11132,7 @@
       <c r="C136">
         <v>2026</v>
       </c>
-      <c r="D136" s="2">
+      <c r="D136" s="1">
         <v>45952</v>
       </c>
       <c r="F136" t="s">
@@ -11196,7 +11170,7 @@
       <c r="C137">
         <v>2026</v>
       </c>
-      <c r="D137" s="2">
+      <c r="D137" s="1">
         <v>46230</v>
       </c>
       <c r="F137" t="s">
@@ -11269,7 +11243,7 @@
       <c r="C139">
         <v>2026</v>
       </c>
-      <c r="D139" s="2">
+      <c r="D139" s="1">
         <v>46029</v>
       </c>
       <c r="G139" t="s">
@@ -11307,7 +11281,7 @@
       <c r="C140">
         <v>2026</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140" s="1">
         <v>46029</v>
       </c>
       <c r="G140" t="s">
@@ -11377,7 +11351,7 @@
       <c r="C142">
         <v>2026</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142" s="1">
         <v>46119</v>
       </c>
       <c r="F142" t="s">
@@ -11482,7 +11456,7 @@
       <c r="C145">
         <v>2026</v>
       </c>
-      <c r="D145" s="2">
+      <c r="D145" s="1">
         <v>46140</v>
       </c>
       <c r="F145" t="s">
@@ -11523,7 +11497,7 @@
       <c r="C146">
         <v>2026</v>
       </c>
-      <c r="D146" s="2">
+      <c r="D146" s="1">
         <v>46230</v>
       </c>
       <c r="F146" t="s">
@@ -11564,7 +11538,7 @@
       <c r="C147">
         <v>2026</v>
       </c>
-      <c r="D147" s="2">
+      <c r="D147" s="1">
         <v>46230</v>
       </c>
       <c r="F147" t="s">
@@ -11605,7 +11579,7 @@
       <c r="C148">
         <v>2026</v>
       </c>
-      <c r="D148" s="2">
+      <c r="D148" s="1">
         <v>46119</v>
       </c>
       <c r="F148" t="s">
@@ -11646,7 +11620,7 @@
       <c r="C149">
         <v>2026</v>
       </c>
-      <c r="D149" s="2">
+      <c r="D149" s="1">
         <v>46230</v>
       </c>
       <c r="F149" t="s">
@@ -11687,7 +11661,7 @@
       <c r="C150">
         <v>2026</v>
       </c>
-      <c r="D150" s="2">
+      <c r="D150" s="1">
         <v>46140</v>
       </c>
       <c r="F150" t="s">
@@ -11728,7 +11702,7 @@
       <c r="C151">
         <v>2026</v>
       </c>
-      <c r="D151" s="2">
+      <c r="D151" s="1">
         <v>45876</v>
       </c>
       <c r="F151" t="s">
@@ -11801,7 +11775,7 @@
       <c r="C153">
         <v>2026</v>
       </c>
-      <c r="D153" s="2">
+      <c r="D153" s="1">
         <v>45863</v>
       </c>
       <c r="F153" t="s">
@@ -11842,7 +11816,7 @@
       <c r="C154">
         <v>2026</v>
       </c>
-      <c r="D154" s="2">
+      <c r="D154" s="1">
         <v>45863</v>
       </c>
       <c r="F154" t="s">
@@ -11883,7 +11857,7 @@
       <c r="C155">
         <v>2026</v>
       </c>
-      <c r="D155" s="2">
+      <c r="D155" s="1">
         <v>45863</v>
       </c>
       <c r="F155" t="s">
@@ -11924,7 +11898,7 @@
       <c r="C156">
         <v>2026</v>
       </c>
-      <c r="D156" s="2">
+      <c r="D156" s="1">
         <v>45860</v>
       </c>
       <c r="F156" t="s">
@@ -11994,7 +11968,7 @@
       <c r="C158">
         <v>2026</v>
       </c>
-      <c r="D158" s="2">
+      <c r="D158" s="1">
         <v>46119</v>
       </c>
       <c r="F158" t="s">
@@ -12035,7 +12009,7 @@
       <c r="C159">
         <v>2026</v>
       </c>
-      <c r="D159" s="2">
+      <c r="D159" s="1">
         <v>45814</v>
       </c>
       <c r="F159" t="s">
@@ -12076,7 +12050,7 @@
       <c r="C160">
         <v>2026</v>
       </c>
-      <c r="D160" s="2">
+      <c r="D160" s="1">
         <v>45817</v>
       </c>
       <c r="F160" t="s">
@@ -12117,7 +12091,7 @@
       <c r="C161">
         <v>2026</v>
       </c>
-      <c r="D161" s="2">
+      <c r="D161" s="1">
         <v>45971</v>
       </c>
       <c r="F161" t="s">
@@ -12158,7 +12132,7 @@
       <c r="C162">
         <v>2026</v>
       </c>
-      <c r="D162" s="2">
+      <c r="D162" s="1">
         <v>45971</v>
       </c>
       <c r="F162" t="s">
@@ -12199,7 +12173,7 @@
       <c r="C163">
         <v>2026</v>
       </c>
-      <c r="D163" s="2">
+      <c r="D163" s="1">
         <v>45860</v>
       </c>
       <c r="G163" t="s">
@@ -12237,7 +12211,7 @@
       <c r="C164">
         <v>2026</v>
       </c>
-      <c r="D164" s="2">
+      <c r="D164" s="1">
         <v>45856</v>
       </c>
       <c r="F164" t="s">
@@ -12310,7 +12284,7 @@
       <c r="C166">
         <v>2026</v>
       </c>
-      <c r="D166" s="2">
+      <c r="D166" s="1">
         <v>46064</v>
       </c>
       <c r="F166" t="s">
@@ -12351,7 +12325,7 @@
       <c r="C167">
         <v>2026</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D167" s="1">
         <v>45982</v>
       </c>
       <c r="G167" t="s">
@@ -12389,7 +12363,7 @@
       <c r="C168">
         <v>2026</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D168" s="1">
         <v>46157</v>
       </c>
       <c r="H168" t="s">
@@ -12424,7 +12398,7 @@
       <c r="C169">
         <v>2026</v>
       </c>
-      <c r="D169" s="2">
+      <c r="D169" s="1">
         <v>45762</v>
       </c>
       <c r="F169" t="s">
@@ -12465,7 +12439,7 @@
       <c r="C170">
         <v>2026</v>
       </c>
-      <c r="D170" s="2">
+      <c r="D170" s="1">
         <v>45816</v>
       </c>
       <c r="F170" t="s">
@@ -12506,7 +12480,7 @@
       <c r="C171">
         <v>2026</v>
       </c>
-      <c r="D171" s="2">
+      <c r="D171" s="1">
         <v>45816</v>
       </c>
       <c r="F171" t="s">
@@ -12585,7 +12559,7 @@
       <c r="C173">
         <v>2026</v>
       </c>
-      <c r="D173" s="2">
+      <c r="D173" s="1">
         <v>46101</v>
       </c>
       <c r="F173" t="s">
@@ -12626,7 +12600,7 @@
       <c r="C174">
         <v>2026</v>
       </c>
-      <c r="D174" s="2">
+      <c r="D174" s="1">
         <v>46101</v>
       </c>
       <c r="F174" t="s">
@@ -12667,7 +12641,7 @@
       <c r="C175">
         <v>2026</v>
       </c>
-      <c r="D175" s="2">
+      <c r="D175" s="1">
         <v>46105</v>
       </c>
       <c r="F175" t="s">
@@ -12708,7 +12682,7 @@
       <c r="C176">
         <v>2026</v>
       </c>
-      <c r="D176" s="2">
+      <c r="D176" s="1">
         <v>45889</v>
       </c>
       <c r="F176" t="s">
@@ -12749,7 +12723,7 @@
       <c r="C177">
         <v>2026</v>
       </c>
-      <c r="D177" s="2">
+      <c r="D177" s="1">
         <v>45814</v>
       </c>
       <c r="F177" t="s">
@@ -12790,7 +12764,7 @@
       <c r="C178">
         <v>2026</v>
       </c>
-      <c r="D178" s="2">
+      <c r="D178" s="1">
         <v>45889</v>
       </c>
       <c r="F178" t="s">
@@ -12831,7 +12805,7 @@
       <c r="C179">
         <v>2026</v>
       </c>
-      <c r="D179" s="2">
+      <c r="D179" s="1">
         <v>45814</v>
       </c>
       <c r="F179" t="s">
@@ -12872,7 +12846,7 @@
       <c r="C180">
         <v>2026</v>
       </c>
-      <c r="D180" s="2">
+      <c r="D180" s="1">
         <v>45889</v>
       </c>
       <c r="F180" t="s">
@@ -12945,7 +12919,7 @@
       <c r="C182">
         <v>2026</v>
       </c>
-      <c r="D182" s="2">
+      <c r="D182" s="1">
         <v>46139</v>
       </c>
       <c r="H182" t="s">
@@ -13012,7 +12986,7 @@
       <c r="C184">
         <v>2026</v>
       </c>
-      <c r="D184" s="2">
+      <c r="D184" s="1">
         <v>45889</v>
       </c>
       <c r="F184" t="s">
@@ -13085,7 +13059,7 @@
       <c r="C186">
         <v>2026</v>
       </c>
-      <c r="D186" s="2">
+      <c r="D186" s="1">
         <v>45814</v>
       </c>
       <c r="F186" t="s">
@@ -13126,7 +13100,7 @@
       <c r="C187">
         <v>2026</v>
       </c>
-      <c r="D187" s="2">
+      <c r="D187" s="1">
         <v>45889</v>
       </c>
       <c r="F187" t="s">
@@ -13167,7 +13141,7 @@
       <c r="C188">
         <v>2026</v>
       </c>
-      <c r="D188" s="2">
+      <c r="D188" s="1">
         <v>45931</v>
       </c>
       <c r="F188" t="s">
@@ -13208,7 +13182,7 @@
       <c r="C189">
         <v>2026</v>
       </c>
-      <c r="D189" s="2">
+      <c r="D189" s="1">
         <v>45889</v>
       </c>
       <c r="F189" t="s">
@@ -13249,7 +13223,7 @@
       <c r="C190">
         <v>2026</v>
       </c>
-      <c r="D190" s="2">
+      <c r="D190" s="1">
         <v>45876</v>
       </c>
       <c r="F190" t="s">
@@ -13290,7 +13264,7 @@
       <c r="C191">
         <v>2026</v>
       </c>
-      <c r="D191" s="2">
+      <c r="D191" s="1">
         <v>45876</v>
       </c>
       <c r="F191" t="s">
@@ -13363,7 +13337,7 @@
       <c r="C193">
         <v>2026</v>
       </c>
-      <c r="D193" s="2">
+      <c r="D193" s="1">
         <v>45876</v>
       </c>
       <c r="F193" t="s">
@@ -13404,7 +13378,7 @@
       <c r="C194">
         <v>2026</v>
       </c>
-      <c r="D194" s="2">
+      <c r="D194" s="1">
         <v>46119</v>
       </c>
       <c r="F194" t="s">
@@ -13445,7 +13419,7 @@
       <c r="C195">
         <v>2026</v>
       </c>
-      <c r="D195" s="2">
+      <c r="D195" s="1">
         <v>46119</v>
       </c>
       <c r="F195" t="s">
@@ -13486,7 +13460,7 @@
       <c r="C196">
         <v>2026</v>
       </c>
-      <c r="D196" s="2">
+      <c r="D196" s="1">
         <v>45961</v>
       </c>
       <c r="F196" t="s">
@@ -13527,7 +13501,7 @@
       <c r="C197">
         <v>2026</v>
       </c>
-      <c r="D197" s="2">
+      <c r="D197" s="1">
         <v>45860</v>
       </c>
       <c r="F197" t="s">
@@ -13568,7 +13542,7 @@
       <c r="C198">
         <v>2026</v>
       </c>
-      <c r="D198" s="2">
+      <c r="D198" s="1">
         <v>45993</v>
       </c>
       <c r="G198" t="s">
@@ -13606,7 +13580,7 @@
       <c r="C199">
         <v>2026</v>
       </c>
-      <c r="D199" s="2">
+      <c r="D199" s="1">
         <v>45853</v>
       </c>
       <c r="F199" t="s">
@@ -13647,7 +13621,7 @@
       <c r="C200">
         <v>2026</v>
       </c>
-      <c r="D200" s="2">
+      <c r="D200" s="1">
         <v>46119</v>
       </c>
       <c r="F200" t="s">
@@ -13726,7 +13700,7 @@
       <c r="C202">
         <v>2026</v>
       </c>
-      <c r="D202" s="2">
+      <c r="D202" s="1">
         <v>46191</v>
       </c>
       <c r="F202" t="s">
@@ -13767,7 +13741,7 @@
       <c r="C203">
         <v>2026</v>
       </c>
-      <c r="D203" s="2">
+      <c r="D203" s="1">
         <v>46191</v>
       </c>
       <c r="F203" t="s">
@@ -13808,7 +13782,7 @@
       <c r="C204">
         <v>2026</v>
       </c>
-      <c r="D204" s="2">
+      <c r="D204" s="1">
         <v>46191</v>
       </c>
       <c r="F204" t="s">
@@ -13849,7 +13823,7 @@
       <c r="C205">
         <v>2026</v>
       </c>
-      <c r="D205" s="2">
+      <c r="D205" s="1">
         <v>45932</v>
       </c>
       <c r="G205" t="s">
@@ -13887,7 +13861,7 @@
       <c r="C206">
         <v>2026</v>
       </c>
-      <c r="D206" s="2">
+      <c r="D206" s="1">
         <v>46191</v>
       </c>
       <c r="F206" t="s">
@@ -13928,7 +13902,7 @@
       <c r="C207">
         <v>2026</v>
       </c>
-      <c r="D207" s="2">
+      <c r="D207" s="1">
         <v>46119</v>
       </c>
       <c r="F207" t="s">
@@ -13969,7 +13943,7 @@
       <c r="C208">
         <v>2026</v>
       </c>
-      <c r="D208" s="2">
+      <c r="D208" s="1">
         <v>45946</v>
       </c>
       <c r="G208" t="s">
@@ -14007,7 +13981,7 @@
       <c r="C209">
         <v>2026</v>
       </c>
-      <c r="D209" s="2">
+      <c r="D209" s="1">
         <v>45937</v>
       </c>
       <c r="F209" t="s">
@@ -14048,7 +14022,7 @@
       <c r="C210">
         <v>2026</v>
       </c>
-      <c r="D210" s="2">
+      <c r="D210" s="1">
         <v>45849</v>
       </c>
       <c r="F210" t="s">
@@ -14089,7 +14063,7 @@
       <c r="C211">
         <v>2026</v>
       </c>
-      <c r="D211" s="2">
+      <c r="D211" s="1">
         <v>45876</v>
       </c>
       <c r="F211" t="s">
@@ -14130,7 +14104,7 @@
       <c r="C212">
         <v>2026</v>
       </c>
-      <c r="D212" s="2">
+      <c r="D212" s="1">
         <v>46008</v>
       </c>
       <c r="F212" t="s">
@@ -14244,7 +14218,7 @@
       <c r="C215">
         <v>2026</v>
       </c>
-      <c r="D215" s="2">
+      <c r="D215" s="1">
         <v>45973</v>
       </c>
       <c r="F215" t="s">
@@ -14285,7 +14259,7 @@
       <c r="C216">
         <v>2026</v>
       </c>
-      <c r="D216" s="2">
+      <c r="D216" s="1">
         <v>46014</v>
       </c>
       <c r="F216" t="s">
@@ -14326,7 +14300,7 @@
       <c r="C217">
         <v>2026</v>
       </c>
-      <c r="D217" s="2">
+      <c r="D217" s="1">
         <v>45876</v>
       </c>
       <c r="F217" t="s">
@@ -14367,7 +14341,7 @@
       <c r="C218">
         <v>2026</v>
       </c>
-      <c r="D218" s="2">
+      <c r="D218" s="1">
         <v>45937</v>
       </c>
       <c r="F218" t="s">
@@ -14408,7 +14382,7 @@
       <c r="C219">
         <v>2026</v>
       </c>
-      <c r="D219" s="2">
+      <c r="D219" s="1">
         <v>45980</v>
       </c>
       <c r="F219" t="s">
@@ -14769,7 +14743,7 @@
       <c r="C230">
         <v>2026</v>
       </c>
-      <c r="D230" s="2">
+      <c r="D230" s="1">
         <v>45979</v>
       </c>
       <c r="F230" t="s">
@@ -14810,7 +14784,7 @@
       <c r="C231">
         <v>2026</v>
       </c>
-      <c r="D231" s="2">
+      <c r="D231" s="1">
         <v>45979</v>
       </c>
       <c r="F231" t="s">
@@ -14851,7 +14825,7 @@
       <c r="C232">
         <v>2026</v>
       </c>
-      <c r="D232" s="2">
+      <c r="D232" s="1">
         <v>45979</v>
       </c>
       <c r="F232" t="s">
@@ -14892,7 +14866,7 @@
       <c r="C233">
         <v>2026</v>
       </c>
-      <c r="D233" s="2">
+      <c r="D233" s="1">
         <v>45971</v>
       </c>
       <c r="F233" t="s">
@@ -14933,7 +14907,7 @@
       <c r="C234">
         <v>2026</v>
       </c>
-      <c r="D234" s="2">
+      <c r="D234" s="1">
         <v>45971</v>
       </c>
       <c r="F234" t="s">
@@ -14974,7 +14948,7 @@
       <c r="C235">
         <v>2026</v>
       </c>
-      <c r="D235" s="2">
+      <c r="D235" s="1">
         <v>45971</v>
       </c>
       <c r="F235" t="s">
@@ -15015,7 +14989,7 @@
       <c r="C236">
         <v>2026</v>
       </c>
-      <c r="D236" s="2">
+      <c r="D236" s="1">
         <v>45889</v>
       </c>
       <c r="F236" t="s">
@@ -15152,7 +15126,7 @@
       <c r="C240">
         <v>2026</v>
       </c>
-      <c r="D240" s="2">
+      <c r="D240" s="1">
         <v>45859</v>
       </c>
       <c r="F240" t="s">
@@ -15193,7 +15167,7 @@
       <c r="C241">
         <v>2026</v>
       </c>
-      <c r="D241" s="2">
+      <c r="D241" s="1">
         <v>45918</v>
       </c>
       <c r="F241" t="s">
@@ -15266,7 +15240,7 @@
       <c r="C243">
         <v>2026</v>
       </c>
-      <c r="D243" s="2">
+      <c r="D243" s="1">
         <v>45874</v>
       </c>
       <c r="F243" t="s">
@@ -15307,7 +15281,7 @@
       <c r="C244">
         <v>2026</v>
       </c>
-      <c r="D244" s="2">
+      <c r="D244" s="1">
         <v>45975</v>
       </c>
       <c r="F244" t="s">
@@ -15345,7 +15319,7 @@
       <c r="C245">
         <v>2026</v>
       </c>
-      <c r="D245" s="2">
+      <c r="D245" s="1">
         <v>45975</v>
       </c>
       <c r="F245" t="s">
@@ -15383,7 +15357,7 @@
       <c r="C246">
         <v>2026</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D246" s="1">
         <v>45975</v>
       </c>
       <c r="F246" t="s">
@@ -15645,7 +15619,7 @@
       <c r="C254">
         <v>2026</v>
       </c>
-      <c r="D254" s="2">
+      <c r="D254" s="1">
         <v>46119</v>
       </c>
       <c r="F254" t="s">
@@ -15750,7 +15724,7 @@
       <c r="C257">
         <v>2026</v>
       </c>
-      <c r="D257" s="2">
+      <c r="D257" s="1">
         <v>45802</v>
       </c>
       <c r="F257" t="s">
@@ -15791,7 +15765,7 @@
       <c r="C258">
         <v>2026</v>
       </c>
-      <c r="D258" s="2">
+      <c r="D258" s="1">
         <v>45804</v>
       </c>
       <c r="F258" t="s">
@@ -15832,7 +15806,7 @@
       <c r="C259">
         <v>2026</v>
       </c>
-      <c r="D259" s="2">
+      <c r="D259" s="1">
         <v>46097</v>
       </c>
       <c r="F259" t="s">
@@ -15873,7 +15847,7 @@
       <c r="C260">
         <v>2026</v>
       </c>
-      <c r="D260" s="2">
+      <c r="D260" s="1">
         <v>45860</v>
       </c>
       <c r="G260" t="s">
@@ -15911,7 +15885,7 @@
       <c r="C261">
         <v>2026</v>
       </c>
-      <c r="D261" s="2">
+      <c r="D261" s="1">
         <v>45889</v>
       </c>
       <c r="F261" t="s">
@@ -15952,7 +15926,7 @@
       <c r="C262">
         <v>2026</v>
       </c>
-      <c r="D262" s="2">
+      <c r="D262" s="1">
         <v>45744</v>
       </c>
       <c r="F262" t="s">
@@ -15993,7 +15967,7 @@
       <c r="C263">
         <v>2026</v>
       </c>
-      <c r="D263" s="2">
+      <c r="D263" s="1">
         <v>45744</v>
       </c>
       <c r="F263" t="s">
@@ -16034,7 +16008,7 @@
       <c r="C264">
         <v>2026</v>
       </c>
-      <c r="D264" s="2">
+      <c r="D264" s="1">
         <v>46408</v>
       </c>
       <c r="F264" t="s">
@@ -16078,7 +16052,7 @@
       <c r="C265">
         <v>2026</v>
       </c>
-      <c r="D265" s="2">
+      <c r="D265" s="1">
         <v>45898</v>
       </c>
       <c r="F265" t="s">
@@ -16119,7 +16093,7 @@
       <c r="C266">
         <v>2026</v>
       </c>
-      <c r="D266" s="2">
+      <c r="D266" s="1">
         <v>45971</v>
       </c>
       <c r="F266" t="s">
@@ -16160,7 +16134,7 @@
       <c r="C267">
         <v>2026</v>
       </c>
-      <c r="D267" s="2">
+      <c r="D267" s="1">
         <v>45744</v>
       </c>
       <c r="F267" t="s">
@@ -16201,7 +16175,7 @@
       <c r="C268">
         <v>2026</v>
       </c>
-      <c r="D268" s="2">
+      <c r="D268" s="1">
         <v>46092</v>
       </c>
       <c r="F268" t="s">
@@ -16242,7 +16216,7 @@
       <c r="C269">
         <v>2026</v>
       </c>
-      <c r="D269" s="2">
+      <c r="D269" s="1">
         <v>46204</v>
       </c>
       <c r="F269" t="s">
@@ -16286,7 +16260,7 @@
       <c r="C270">
         <v>2026</v>
       </c>
-      <c r="D270" s="2">
+      <c r="D270" s="1">
         <v>46185</v>
       </c>
       <c r="H270" t="s">
@@ -16321,7 +16295,7 @@
       <c r="C271">
         <v>2026</v>
       </c>
-      <c r="D271" s="2">
+      <c r="D271" s="1">
         <v>45890</v>
       </c>
       <c r="G271" t="s">
@@ -16359,7 +16333,7 @@
       <c r="C272">
         <v>2026</v>
       </c>
-      <c r="D272" s="2">
+      <c r="D272" s="1">
         <v>46185</v>
       </c>
       <c r="H272" t="s">
@@ -16394,7 +16368,7 @@
       <c r="C273">
         <v>2026</v>
       </c>
-      <c r="D273" s="2">
+      <c r="D273" s="1">
         <v>46175</v>
       </c>
       <c r="F273" t="s">
@@ -16435,7 +16409,7 @@
       <c r="C274">
         <v>2026</v>
       </c>
-      <c r="D274" s="2">
+      <c r="D274" s="1">
         <v>45890</v>
       </c>
       <c r="G274" t="s">
@@ -16473,7 +16447,7 @@
       <c r="C275">
         <v>2026</v>
       </c>
-      <c r="D275" s="2">
+      <c r="D275" s="1">
         <v>46175</v>
       </c>
       <c r="F275" t="s">
@@ -16514,7 +16488,7 @@
       <c r="C276">
         <v>2026</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D276" s="1">
         <v>46185</v>
       </c>
       <c r="G276" t="s">
@@ -16552,7 +16526,7 @@
       <c r="C277">
         <v>2026</v>
       </c>
-      <c r="D277" s="2">
+      <c r="D277" s="1">
         <v>45890</v>
       </c>
       <c r="G277" t="s">
@@ -16590,7 +16564,7 @@
       <c r="C278">
         <v>2026</v>
       </c>
-      <c r="D278" s="2">
+      <c r="D278" s="1">
         <v>45890</v>
       </c>
       <c r="G278" t="s">
@@ -16628,7 +16602,7 @@
       <c r="C279">
         <v>2026</v>
       </c>
-      <c r="D279" s="2">
+      <c r="D279" s="1">
         <v>45890</v>
       </c>
       <c r="G279" t="s">
@@ -16666,7 +16640,7 @@
       <c r="C280">
         <v>2026</v>
       </c>
-      <c r="D280" s="2">
+      <c r="D280" s="1">
         <v>46175</v>
       </c>
       <c r="F280" t="s">
@@ -16707,7 +16681,7 @@
       <c r="C281">
         <v>2026</v>
       </c>
-      <c r="D281" s="2">
+      <c r="D281" s="1">
         <v>45890</v>
       </c>
       <c r="G281" t="s">
@@ -16745,7 +16719,7 @@
       <c r="C282">
         <v>2026</v>
       </c>
-      <c r="D282" s="2">
+      <c r="D282" s="1">
         <v>46119</v>
       </c>
       <c r="F282" t="s">
@@ -16786,7 +16760,7 @@
       <c r="C283">
         <v>2026</v>
       </c>
-      <c r="D283" s="2">
+      <c r="D283" s="1">
         <v>46119</v>
       </c>
       <c r="F283" t="s">
@@ -16827,7 +16801,7 @@
       <c r="C284">
         <v>2026</v>
       </c>
-      <c r="D284" s="2">
+      <c r="D284" s="1">
         <v>46119</v>
       </c>
       <c r="F284" t="s">
@@ -16932,7 +16906,7 @@
       <c r="C287">
         <v>2026</v>
       </c>
-      <c r="D287" s="2">
+      <c r="D287" s="1">
         <v>45856</v>
       </c>
       <c r="F287" t="s">
@@ -16973,7 +16947,7 @@
       <c r="C288">
         <v>2026</v>
       </c>
-      <c r="D288" s="2">
+      <c r="D288" s="1">
         <v>45769</v>
       </c>
       <c r="F288" t="s">
@@ -17014,7 +16988,7 @@
       <c r="C289">
         <v>2026</v>
       </c>
-      <c r="D289" s="2">
+      <c r="D289" s="1">
         <v>45769</v>
       </c>
       <c r="F289" t="s">
@@ -17055,7 +17029,7 @@
       <c r="C290">
         <v>2026</v>
       </c>
-      <c r="D290" s="2">
+      <c r="D290" s="1">
         <v>45769</v>
       </c>
       <c r="F290" t="s">
@@ -17096,7 +17070,7 @@
       <c r="C291">
         <v>2026</v>
       </c>
-      <c r="D291" s="2">
+      <c r="D291" s="1">
         <v>45769</v>
       </c>
       <c r="F291" t="s">
@@ -17137,7 +17111,7 @@
       <c r="C292">
         <v>2026</v>
       </c>
-      <c r="D292" s="2">
+      <c r="D292" s="1">
         <v>45769</v>
       </c>
       <c r="F292" t="s">
@@ -17178,7 +17152,7 @@
       <c r="C293">
         <v>2026</v>
       </c>
-      <c r="D293" s="2">
+      <c r="D293" s="1">
         <v>45769</v>
       </c>
       <c r="F293" t="s">
@@ -17219,7 +17193,7 @@
       <c r="C294">
         <v>2026</v>
       </c>
-      <c r="D294" s="2">
+      <c r="D294" s="1">
         <v>45769</v>
       </c>
       <c r="F294" t="s">
@@ -17260,7 +17234,7 @@
       <c r="C295">
         <v>2026</v>
       </c>
-      <c r="D295" s="2">
+      <c r="D295" s="1">
         <v>46147</v>
       </c>
       <c r="H295" t="s">
@@ -17295,7 +17269,7 @@
       <c r="C296">
         <v>2026</v>
       </c>
-      <c r="D296" s="2">
+      <c r="D296" s="1">
         <v>46147</v>
       </c>
       <c r="H296" t="s">
@@ -17330,7 +17304,7 @@
       <c r="C297">
         <v>2026</v>
       </c>
-      <c r="D297" s="2">
+      <c r="D297" s="1">
         <v>46147</v>
       </c>
       <c r="H297" t="s">
@@ -17365,7 +17339,7 @@
       <c r="C298">
         <v>2026</v>
       </c>
-      <c r="D298" s="2">
+      <c r="D298" s="1">
         <v>45814</v>
       </c>
       <c r="F298" t="s">
@@ -17438,7 +17412,7 @@
       <c r="C300">
         <v>2026</v>
       </c>
-      <c r="D300" s="2">
+      <c r="D300" s="1">
         <v>45860</v>
       </c>
       <c r="F300" t="s">
@@ -17479,7 +17453,7 @@
       <c r="C301">
         <v>2026</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>45971</v>
       </c>
       <c r="F301" t="s">
@@ -17520,7 +17494,7 @@
       <c r="C302">
         <v>2026</v>
       </c>
-      <c r="D302" s="2">
+      <c r="D302" s="1">
         <v>45863</v>
       </c>
       <c r="F302" t="s">
@@ -17561,7 +17535,7 @@
       <c r="C303">
         <v>2026</v>
       </c>
-      <c r="D303" s="2">
+      <c r="D303" s="1">
         <v>45905</v>
       </c>
       <c r="G303" t="s">
@@ -17599,7 +17573,7 @@
       <c r="C304">
         <v>2026</v>
       </c>
-      <c r="D304" s="2">
+      <c r="D304" s="1">
         <v>45971</v>
       </c>
       <c r="F304" t="s">
@@ -17640,7 +17614,7 @@
       <c r="C305">
         <v>2026</v>
       </c>
-      <c r="D305" s="2">
+      <c r="D305" s="1">
         <v>45971</v>
       </c>
       <c r="F305" t="s">
@@ -17681,7 +17655,7 @@
       <c r="C306">
         <v>2026</v>
       </c>
-      <c r="D306" s="2">
+      <c r="D306" s="1">
         <v>45744</v>
       </c>
       <c r="F306" t="s">
@@ -17722,7 +17696,7 @@
       <c r="C307">
         <v>2026</v>
       </c>
-      <c r="D307" s="2">
+      <c r="D307" s="1">
         <v>45814</v>
       </c>
       <c r="F307" t="s">
@@ -17763,7 +17737,7 @@
       <c r="C308">
         <v>2026</v>
       </c>
-      <c r="D308" s="2">
+      <c r="D308" s="1">
         <v>45807</v>
       </c>
       <c r="F308" t="s">
@@ -17804,7 +17778,7 @@
       <c r="C309">
         <v>2026</v>
       </c>
-      <c r="D309" s="2">
+      <c r="D309" s="1">
         <v>45802</v>
       </c>
       <c r="F309" t="s">
@@ -17845,7 +17819,7 @@
       <c r="C310">
         <v>2026</v>
       </c>
-      <c r="D310" s="2">
+      <c r="D310" s="1">
         <v>45802</v>
       </c>
       <c r="F310" t="s">
@@ -17886,7 +17860,7 @@
       <c r="C311">
         <v>2026</v>
       </c>
-      <c r="D311" s="2">
+      <c r="D311" s="1">
         <v>45802</v>
       </c>
       <c r="F311" t="s">
@@ -17927,7 +17901,7 @@
       <c r="C312">
         <v>2026</v>
       </c>
-      <c r="D312" s="2">
+      <c r="D312" s="1">
         <v>45897</v>
       </c>
       <c r="H312" t="s">
@@ -17962,7 +17936,7 @@
       <c r="C313">
         <v>2026</v>
       </c>
-      <c r="D313" s="2">
+      <c r="D313" s="1">
         <v>45802</v>
       </c>
       <c r="F313" t="s">
@@ -18003,7 +17977,7 @@
       <c r="C314">
         <v>2026</v>
       </c>
-      <c r="D314" s="2">
+      <c r="D314" s="1">
         <v>45802</v>
       </c>
       <c r="F314" t="s">
@@ -18044,7 +18018,7 @@
       <c r="C315">
         <v>2026</v>
       </c>
-      <c r="D315" s="2">
+      <c r="D315" s="1">
         <v>45876</v>
       </c>
       <c r="F315" t="s">
@@ -18085,7 +18059,7 @@
       <c r="C316">
         <v>2026</v>
       </c>
-      <c r="D316" s="2">
+      <c r="D316" s="1">
         <v>45889</v>
       </c>
       <c r="F316" t="s">
@@ -18126,7 +18100,7 @@
       <c r="C317">
         <v>2026</v>
       </c>
-      <c r="D317" s="2">
+      <c r="D317" s="1">
         <v>45876</v>
       </c>
       <c r="F317" t="s">
@@ -18167,7 +18141,7 @@
       <c r="C318">
         <v>2026</v>
       </c>
-      <c r="D318" s="2">
+      <c r="D318" s="1">
         <v>45926</v>
       </c>
       <c r="F318" t="s">
@@ -18208,7 +18182,7 @@
       <c r="C319">
         <v>2026</v>
       </c>
-      <c r="D319" s="2">
+      <c r="D319" s="1">
         <v>45909</v>
       </c>
       <c r="F319" t="s">
@@ -18249,7 +18223,7 @@
       <c r="C320">
         <v>2026</v>
       </c>
-      <c r="D320" s="2">
+      <c r="D320" s="1">
         <v>46119</v>
       </c>
       <c r="F320" t="s">
@@ -18354,7 +18328,7 @@
       <c r="C323">
         <v>2026</v>
       </c>
-      <c r="D323" s="2">
+      <c r="D323" s="1">
         <v>46119</v>
       </c>
       <c r="F323" t="s">
@@ -18395,7 +18369,7 @@
       <c r="C324">
         <v>2026</v>
       </c>
-      <c r="D324" s="2">
+      <c r="D324" s="1">
         <v>46119</v>
       </c>
       <c r="F324" t="s">
@@ -18532,7 +18506,7 @@
       <c r="C328">
         <v>2026</v>
       </c>
-      <c r="D328" s="2">
+      <c r="D328" s="1">
         <v>46086</v>
       </c>
       <c r="G328" t="s">
@@ -18602,7 +18576,7 @@
       <c r="C330">
         <v>2026</v>
       </c>
-      <c r="D330" s="2">
+      <c r="D330" s="1">
         <v>45965</v>
       </c>
       <c r="F330" t="s">
@@ -18643,7 +18617,7 @@
       <c r="C331">
         <v>2026</v>
       </c>
-      <c r="D331" s="2">
+      <c r="D331" s="1">
         <v>46064</v>
       </c>
       <c r="H331" t="s">
@@ -18675,7 +18649,7 @@
       <c r="C332">
         <v>2026</v>
       </c>
-      <c r="D332" s="2">
+      <c r="D332" s="1">
         <v>46049</v>
       </c>
       <c r="F332" t="s">
@@ -18716,7 +18690,7 @@
       <c r="C333">
         <v>2026</v>
       </c>
-      <c r="D333" s="2">
+      <c r="D333" s="1">
         <v>45996</v>
       </c>
       <c r="G333" t="s">
@@ -18754,7 +18728,7 @@
       <c r="C334">
         <v>2026</v>
       </c>
-      <c r="D334" s="2">
+      <c r="D334" s="1">
         <v>45996</v>
       </c>
       <c r="G334" t="s">
@@ -18792,7 +18766,7 @@
       <c r="C335">
         <v>2026</v>
       </c>
-      <c r="D335" s="2">
+      <c r="D335" s="1">
         <v>45989</v>
       </c>
       <c r="G335" t="s">
@@ -18830,7 +18804,7 @@
       <c r="C336">
         <v>2026</v>
       </c>
-      <c r="D336" s="2">
+      <c r="D336" s="1">
         <v>46156</v>
       </c>
       <c r="H336" t="s">
@@ -18865,7 +18839,7 @@
       <c r="C337">
         <v>2026</v>
       </c>
-      <c r="D337" s="2">
+      <c r="D337" s="1">
         <v>45996</v>
       </c>
       <c r="G337" t="s">
@@ -18903,7 +18877,7 @@
       <c r="C338">
         <v>2026</v>
       </c>
-      <c r="D338" s="2">
+      <c r="D338" s="1">
         <v>45989</v>
       </c>
       <c r="G338" t="s">
@@ -18941,7 +18915,7 @@
       <c r="C339">
         <v>2026</v>
       </c>
-      <c r="D339" s="2">
+      <c r="D339" s="1">
         <v>46002</v>
       </c>
       <c r="G339" t="s">
@@ -18979,7 +18953,7 @@
       <c r="C340">
         <v>2026</v>
       </c>
-      <c r="D340" s="2">
+      <c r="D340" s="1">
         <v>46002</v>
       </c>
       <c r="G340" t="s">
@@ -19017,7 +18991,7 @@
       <c r="C341">
         <v>2026</v>
       </c>
-      <c r="D341" s="2">
+      <c r="D341" s="1">
         <v>45996</v>
       </c>
       <c r="G341" t="s">
@@ -19055,7 +19029,7 @@
       <c r="C342">
         <v>2026</v>
       </c>
-      <c r="D342" s="2">
+      <c r="D342" s="1">
         <v>46002</v>
       </c>
       <c r="G342" t="s">
@@ -19093,7 +19067,7 @@
       <c r="C343">
         <v>2026</v>
       </c>
-      <c r="D343" s="2">
+      <c r="D343" s="1">
         <v>46031</v>
       </c>
       <c r="G343" t="s">
@@ -19131,7 +19105,7 @@
       <c r="C344">
         <v>2026</v>
       </c>
-      <c r="D344" s="2">
+      <c r="D344" s="1">
         <v>46153</v>
       </c>
       <c r="F344" t="s">
@@ -19172,7 +19146,7 @@
       <c r="C345">
         <v>2026</v>
       </c>
-      <c r="D345" s="2">
+      <c r="D345" s="1">
         <v>46135</v>
       </c>
       <c r="F345" t="s">
@@ -19277,7 +19251,7 @@
       <c r="C348">
         <v>2026</v>
       </c>
-      <c r="D348" s="2">
+      <c r="D348" s="1">
         <v>46230</v>
       </c>
       <c r="F348" t="s">
@@ -19382,7 +19356,7 @@
       <c r="C351">
         <v>2026</v>
       </c>
-      <c r="D351" s="2">
+      <c r="D351" s="1">
         <v>45996</v>
       </c>
       <c r="G351" t="s">
@@ -19420,7 +19394,7 @@
       <c r="C352">
         <v>2026</v>
       </c>
-      <c r="D352" s="2">
+      <c r="D352" s="1">
         <v>45996</v>
       </c>
       <c r="G352" t="s">
@@ -19490,7 +19464,7 @@
       <c r="C354">
         <v>2026</v>
       </c>
-      <c r="D354" s="2">
+      <c r="D354" s="1">
         <v>46164</v>
       </c>
       <c r="H354" t="s">
@@ -19525,7 +19499,7 @@
       <c r="C355">
         <v>2026</v>
       </c>
-      <c r="D355" s="2">
+      <c r="D355" s="1">
         <v>46020</v>
       </c>
       <c r="G355" t="s">
@@ -19563,7 +19537,7 @@
       <c r="C356">
         <v>2026</v>
       </c>
-      <c r="D356" s="2">
+      <c r="D356" s="1">
         <v>46225</v>
       </c>
       <c r="F356" t="s">
@@ -19607,7 +19581,7 @@
       <c r="C357">
         <v>2026</v>
       </c>
-      <c r="D357" s="2">
+      <c r="D357" s="1">
         <v>46176</v>
       </c>
       <c r="H357" t="s">
@@ -19642,7 +19616,7 @@
       <c r="C358">
         <v>2026</v>
       </c>
-      <c r="D358" s="2">
+      <c r="D358" s="1">
         <v>46086</v>
       </c>
       <c r="G358" t="s">
@@ -19680,7 +19654,7 @@
       <c r="C359">
         <v>2026</v>
       </c>
-      <c r="D359" s="2">
+      <c r="D359" s="1">
         <v>46052</v>
       </c>
       <c r="G359" t="s">
@@ -19756,7 +19730,7 @@
       <c r="C361">
         <v>2026</v>
       </c>
-      <c r="D361" s="2">
+      <c r="D361" s="1">
         <v>46010</v>
       </c>
       <c r="G361" t="s">
@@ -19794,7 +19768,7 @@
       <c r="C362">
         <v>2026</v>
       </c>
-      <c r="D362" s="2">
+      <c r="D362" s="1">
         <v>46010</v>
       </c>
       <c r="G362" t="s">
@@ -19864,7 +19838,7 @@
       <c r="C364">
         <v>2026</v>
       </c>
-      <c r="D364" s="2">
+      <c r="D364" s="1">
         <v>46079</v>
       </c>
       <c r="F364" t="s">
@@ -19905,7 +19879,7 @@
       <c r="C365">
         <v>2026</v>
       </c>
-      <c r="D365" s="2">
+      <c r="D365" s="1">
         <v>46010</v>
       </c>
       <c r="G365" t="s">
@@ -19943,7 +19917,7 @@
       <c r="C366">
         <v>2026</v>
       </c>
-      <c r="D366" s="2">
+      <c r="D366" s="1">
         <v>46010</v>
       </c>
       <c r="G366" t="s">
@@ -19981,7 +19955,7 @@
       <c r="C367">
         <v>2026</v>
       </c>
-      <c r="D367" s="2">
+      <c r="D367" s="1">
         <v>46230</v>
       </c>
       <c r="F367" t="s">
@@ -20025,7 +19999,7 @@
       <c r="C368">
         <v>2026</v>
       </c>
-      <c r="D368" s="2">
+      <c r="D368" s="1">
         <v>46063</v>
       </c>
       <c r="G368" t="s">
@@ -20063,7 +20037,7 @@
       <c r="C369">
         <v>2026</v>
       </c>
-      <c r="D369" s="2">
+      <c r="D369" s="1">
         <v>46063</v>
       </c>
       <c r="F369" t="s">
@@ -20104,7 +20078,7 @@
       <c r="C370">
         <v>2026</v>
       </c>
-      <c r="D370" s="2">
+      <c r="D370" s="1">
         <v>46063</v>
       </c>
       <c r="F370" t="s">
@@ -20145,7 +20119,7 @@
       <c r="C371">
         <v>2026</v>
       </c>
-      <c r="D371" s="2">
+      <c r="D371" s="1">
         <v>46063</v>
       </c>
       <c r="F371" t="s">
@@ -20186,7 +20160,7 @@
       <c r="C372">
         <v>2026</v>
       </c>
-      <c r="D372" s="2">
+      <c r="D372" s="1">
         <v>46063</v>
       </c>
       <c r="G372" t="s">
@@ -20352,7 +20326,7 @@
       <c r="C377">
         <v>2026</v>
       </c>
-      <c r="D377" s="2">
+      <c r="D377" s="1">
         <v>46114</v>
       </c>
       <c r="F377" t="s">
@@ -20393,7 +20367,7 @@
       <c r="C378">
         <v>2026</v>
       </c>
-      <c r="D378" s="2">
+      <c r="D378" s="1">
         <v>46191</v>
       </c>
       <c r="F378" t="s">
@@ -20434,7 +20408,7 @@
       <c r="C379">
         <v>2026</v>
       </c>
-      <c r="D379" s="2">
+      <c r="D379" s="1">
         <v>46230</v>
       </c>
       <c r="F379" t="s">
@@ -20475,7 +20449,7 @@
       <c r="C380">
         <v>2026</v>
       </c>
-      <c r="D380" s="2">
+      <c r="D380" s="1">
         <v>46230</v>
       </c>
       <c r="F380" t="s">
@@ -20516,7 +20490,7 @@
       <c r="C381">
         <v>2026</v>
       </c>
-      <c r="D381" s="2">
+      <c r="D381" s="1">
         <v>46230</v>
       </c>
       <c r="F381" t="s">
@@ -20557,7 +20531,7 @@
       <c r="C382">
         <v>2026</v>
       </c>
-      <c r="D382" s="2">
+      <c r="D382" s="1">
         <v>46230</v>
       </c>
       <c r="F382" t="s">
@@ -20598,7 +20572,7 @@
       <c r="C383">
         <v>2026</v>
       </c>
-      <c r="D383" s="2">
+      <c r="D383" s="1">
         <v>46230</v>
       </c>
       <c r="F383" t="s">
@@ -20639,7 +20613,7 @@
       <c r="C384">
         <v>2026</v>
       </c>
-      <c r="D384" s="2">
+      <c r="D384" s="1">
         <v>46230</v>
       </c>
       <c r="F384" t="s">
@@ -20680,7 +20654,7 @@
       <c r="C385">
         <v>2026</v>
       </c>
-      <c r="D385" s="2">
+      <c r="D385" s="1">
         <v>46230</v>
       </c>
       <c r="F385" t="s">
@@ -20753,7 +20727,7 @@
       <c r="C387">
         <v>2026</v>
       </c>
-      <c r="D387" s="2">
+      <c r="D387" s="1">
         <v>45996</v>
       </c>
       <c r="G387" t="s">
@@ -20983,7 +20957,7 @@
       <c r="C394">
         <v>2026</v>
       </c>
-      <c r="D394" s="2">
+      <c r="D394" s="1">
         <v>46052</v>
       </c>
       <c r="F394" t="s">
@@ -21024,7 +20998,7 @@
       <c r="C395">
         <v>2026</v>
       </c>
-      <c r="D395" s="2">
+      <c r="D395" s="1">
         <v>46057</v>
       </c>
       <c r="F395" t="s">
@@ -21065,7 +21039,7 @@
       <c r="C396">
         <v>2026</v>
       </c>
-      <c r="D396" s="2">
+      <c r="D396" s="1">
         <v>46112</v>
       </c>
       <c r="F396" t="s">
@@ -21138,7 +21112,7 @@
       <c r="C398">
         <v>2026</v>
       </c>
-      <c r="D398" s="2">
+      <c r="D398" s="1">
         <v>46063</v>
       </c>
       <c r="G398" t="s">
@@ -21176,7 +21150,7 @@
       <c r="C399">
         <v>2026</v>
       </c>
-      <c r="D399" s="2">
+      <c r="D399" s="1">
         <v>46048</v>
       </c>
       <c r="G399" t="s">
@@ -21214,7 +21188,7 @@
       <c r="C400">
         <v>2026</v>
       </c>
-      <c r="D400" s="2">
+      <c r="D400" s="1">
         <v>46063</v>
       </c>
       <c r="H400" t="s">
@@ -21281,7 +21255,7 @@
       <c r="C402">
         <v>2026</v>
       </c>
-      <c r="D402" s="2">
+      <c r="D402" s="1">
         <v>46119</v>
       </c>
       <c r="F402" t="s">
@@ -21354,7 +21328,7 @@
       <c r="C404">
         <v>2026</v>
       </c>
-      <c r="D404" s="2">
+      <c r="D404" s="1">
         <v>46119</v>
       </c>
       <c r="F404" t="s">
@@ -21395,7 +21369,7 @@
       <c r="C405">
         <v>2026</v>
       </c>
-      <c r="D405" s="2">
+      <c r="D405" s="1">
         <v>46113</v>
       </c>
       <c r="F405" t="s">
@@ -21436,7 +21410,7 @@
       <c r="C406">
         <v>2026</v>
       </c>
-      <c r="D406" s="2">
+      <c r="D406" s="1">
         <v>46104</v>
       </c>
       <c r="F406" t="s">
@@ -21477,7 +21451,7 @@
       <c r="C407">
         <v>2026</v>
       </c>
-      <c r="D407" s="2">
+      <c r="D407" s="1">
         <v>46135</v>
       </c>
       <c r="H407" t="s">
@@ -21544,7 +21518,7 @@
       <c r="C409">
         <v>2026</v>
       </c>
-      <c r="D409" s="2">
+      <c r="D409" s="1">
         <v>46230</v>
       </c>
       <c r="F409" t="s">
@@ -21585,7 +21559,7 @@
       <c r="C410">
         <v>2026</v>
       </c>
-      <c r="D410" s="2">
+      <c r="D410" s="1">
         <v>46086</v>
       </c>
       <c r="G410" t="s">
@@ -21623,7 +21597,7 @@
       <c r="C411">
         <v>2026</v>
       </c>
-      <c r="D411" s="2">
+      <c r="D411" s="1">
         <v>46086</v>
       </c>
       <c r="G411" t="s">
@@ -21661,7 +21635,7 @@
       <c r="C412">
         <v>2026</v>
       </c>
-      <c r="D412" s="2">
+      <c r="D412" s="1">
         <v>46086</v>
       </c>
       <c r="H412" t="s">
@@ -21696,7 +21670,7 @@
       <c r="C413">
         <v>2026</v>
       </c>
-      <c r="D413" s="2">
+      <c r="D413" s="1">
         <v>46230</v>
       </c>
       <c r="F413" t="s">
@@ -21833,7 +21807,7 @@
       <c r="C417">
         <v>2026</v>
       </c>
-      <c r="D417" s="2">
+      <c r="D417" s="1">
         <v>46176</v>
       </c>
       <c r="H417" t="s">
@@ -21868,7 +21842,7 @@
       <c r="C418">
         <v>2026</v>
       </c>
-      <c r="D418" s="2">
+      <c r="D418" s="1">
         <v>46147</v>
       </c>
       <c r="H418" t="s">
@@ -21903,7 +21877,7 @@
       <c r="C419">
         <v>2026</v>
       </c>
-      <c r="D419" s="2">
+      <c r="D419" s="1">
         <v>46135</v>
       </c>
       <c r="H419" t="s">
@@ -21970,7 +21944,7 @@
       <c r="C421">
         <v>2026</v>
       </c>
-      <c r="D421" s="2">
+      <c r="D421" s="1">
         <v>46227</v>
       </c>
       <c r="G421" t="s">
@@ -22011,7 +21985,7 @@
       <c r="C422">
         <v>2026</v>
       </c>
-      <c r="D422" s="2">
+      <c r="D422" s="1">
         <v>46230</v>
       </c>
       <c r="F422" t="s">
@@ -22052,7 +22026,7 @@
       <c r="C423">
         <v>2026</v>
       </c>
-      <c r="D423" s="2">
+      <c r="D423" s="1">
         <v>46083</v>
       </c>
       <c r="F423" t="s">
@@ -22093,7 +22067,7 @@
       <c r="C424">
         <v>2026</v>
       </c>
-      <c r="D424" s="2">
+      <c r="D424" s="1">
         <v>46083</v>
       </c>
       <c r="G424" t="s">
@@ -22131,7 +22105,7 @@
       <c r="C425">
         <v>2026</v>
       </c>
-      <c r="D425" s="2">
+      <c r="D425" s="1">
         <v>46083</v>
       </c>
       <c r="F425" t="s">
@@ -22172,7 +22146,7 @@
       <c r="C426">
         <v>2026</v>
       </c>
-      <c r="D426" s="2">
+      <c r="D426" s="1">
         <v>46127</v>
       </c>
       <c r="F426" t="s">
@@ -22213,7 +22187,7 @@
       <c r="C427">
         <v>2026</v>
       </c>
-      <c r="D427" s="2">
+      <c r="D427" s="1">
         <v>46100</v>
       </c>
       <c r="F427" t="s">
@@ -22411,7 +22385,7 @@
       <c r="C433">
         <v>2026</v>
       </c>
-      <c r="D433" s="2">
+      <c r="D433" s="1">
         <v>46230</v>
       </c>
       <c r="F433" t="s">
@@ -22452,7 +22426,7 @@
       <c r="C434">
         <v>2026</v>
       </c>
-      <c r="D434" s="2">
+      <c r="D434" s="1">
         <v>46079</v>
       </c>
       <c r="H434" t="s">
@@ -22583,7 +22557,7 @@
       <c r="C438">
         <v>2026</v>
       </c>
-      <c r="D438" s="2">
+      <c r="D438" s="1">
         <v>46176</v>
       </c>
       <c r="F438" t="s">
@@ -22624,7 +22598,7 @@
       <c r="C439">
         <v>2026</v>
       </c>
-      <c r="D439" s="2">
+      <c r="D439" s="1">
         <v>46176</v>
       </c>
       <c r="F439" t="s">
@@ -22665,7 +22639,7 @@
       <c r="C440">
         <v>2026</v>
       </c>
-      <c r="D440" s="2">
+      <c r="D440" s="1">
         <v>46155</v>
       </c>
       <c r="F440" t="s">
@@ -22706,7 +22680,7 @@
       <c r="C441">
         <v>2026</v>
       </c>
-      <c r="D441" s="2">
+      <c r="D441" s="1">
         <v>46155</v>
       </c>
       <c r="G441" t="s">
@@ -22744,7 +22718,7 @@
       <c r="C442">
         <v>2026</v>
       </c>
-      <c r="D442" s="2">
+      <c r="D442" s="1">
         <v>46129</v>
       </c>
       <c r="F442" t="s">
@@ -22785,7 +22759,7 @@
       <c r="C443">
         <v>2026</v>
       </c>
-      <c r="D443" s="2">
+      <c r="D443" s="1">
         <v>46119</v>
       </c>
       <c r="F443" t="s">
@@ -22826,7 +22800,7 @@
       <c r="C444">
         <v>2026</v>
       </c>
-      <c r="D444" s="2">
+      <c r="D444" s="1">
         <v>46135</v>
       </c>
       <c r="H444" t="s">
@@ -22861,7 +22835,7 @@
       <c r="C445">
         <v>2026</v>
       </c>
-      <c r="D445" s="2">
+      <c r="D445" s="1">
         <v>46127</v>
       </c>
       <c r="H445" t="s">
@@ -22896,7 +22870,7 @@
       <c r="C446">
         <v>2026</v>
       </c>
-      <c r="D446" s="2">
+      <c r="D446" s="1">
         <v>46127</v>
       </c>
       <c r="H446" t="s">
@@ -22963,7 +22937,7 @@
       <c r="C448">
         <v>2026</v>
       </c>
-      <c r="D448" s="2">
+      <c r="D448" s="1">
         <v>46175</v>
       </c>
       <c r="F448" t="s">
@@ -23004,7 +22978,7 @@
       <c r="C449">
         <v>2026</v>
       </c>
-      <c r="D449" s="2">
+      <c r="D449" s="1">
         <v>46139</v>
       </c>
       <c r="H449" t="s">
@@ -23039,7 +23013,7 @@
       <c r="C450">
         <v>2026</v>
       </c>
-      <c r="D450" s="2">
+      <c r="D450" s="1">
         <v>46155</v>
       </c>
       <c r="H450" t="s">
@@ -23074,7 +23048,7 @@
       <c r="C451">
         <v>2026</v>
       </c>
-      <c r="D451" s="2">
+      <c r="D451" s="1">
         <v>46175</v>
       </c>
       <c r="F451" t="s">
@@ -23147,7 +23121,7 @@
       <c r="C453">
         <v>2026</v>
       </c>
-      <c r="D453" s="2">
+      <c r="D453" s="1">
         <v>46156</v>
       </c>
       <c r="F453" t="s">
@@ -23188,7 +23162,7 @@
       <c r="C454">
         <v>2026</v>
       </c>
-      <c r="D454" s="2">
+      <c r="D454" s="1">
         <v>46157</v>
       </c>
       <c r="G454" t="s">
@@ -23226,7 +23200,7 @@
       <c r="C455">
         <v>2026</v>
       </c>
-      <c r="D455" s="2">
+      <c r="D455" s="1">
         <v>46183</v>
       </c>
       <c r="H455" t="s">
@@ -23261,7 +23235,7 @@
       <c r="C456">
         <v>2026</v>
       </c>
-      <c r="D456" s="2">
+      <c r="D456" s="1">
         <v>46183</v>
       </c>
       <c r="H456" t="s">
@@ -23360,7 +23334,7 @@
       <c r="C459">
         <v>2026</v>
       </c>
-      <c r="D459" s="2">
+      <c r="D459" s="1">
         <v>46230</v>
       </c>
       <c r="F459" t="s">
@@ -23404,7 +23378,7 @@
       <c r="C460">
         <v>2026</v>
       </c>
-      <c r="D460" s="2">
+      <c r="D460" s="1">
         <v>46185</v>
       </c>
       <c r="H460" t="s">
@@ -23471,7 +23445,7 @@
       <c r="C462">
         <v>2026</v>
       </c>
-      <c r="D462" s="2">
+      <c r="D462" s="1">
         <v>46185</v>
       </c>
       <c r="H462" t="s">
@@ -23570,7 +23544,7 @@
       <c r="C465">
         <v>2026</v>
       </c>
-      <c r="D465" s="2">
+      <c r="D465" s="1">
         <v>46175</v>
       </c>
       <c r="F465" t="s">
@@ -23611,7 +23585,7 @@
       <c r="C466">
         <v>2026</v>
       </c>
-      <c r="D466" s="2">
+      <c r="D466" s="1">
         <v>46175</v>
       </c>
       <c r="F466" t="s">
@@ -23652,7 +23626,7 @@
       <c r="C467">
         <v>2026</v>
       </c>
-      <c r="D467" s="2">
+      <c r="D467" s="1">
         <v>46230</v>
       </c>
       <c r="F467" t="s">
@@ -23693,7 +23667,7 @@
       <c r="C468">
         <v>2026</v>
       </c>
-      <c r="D468" s="2">
+      <c r="D468" s="1">
         <v>46175</v>
       </c>
       <c r="G468" t="s">
@@ -23731,7 +23705,7 @@
       <c r="C469">
         <v>2026</v>
       </c>
-      <c r="D469" s="2">
+      <c r="D469" s="1">
         <v>46175</v>
       </c>
       <c r="G469" t="s">
@@ -23769,7 +23743,7 @@
       <c r="C470">
         <v>2026</v>
       </c>
-      <c r="D470" s="2">
+      <c r="D470" s="1">
         <v>46175</v>
       </c>
       <c r="G470" t="s">
@@ -23807,7 +23781,7 @@
       <c r="C471">
         <v>2026</v>
       </c>
-      <c r="D471" s="2">
+      <c r="D471" s="1">
         <v>46230</v>
       </c>
       <c r="F471" t="s">
@@ -23848,7 +23822,7 @@
       <c r="C472">
         <v>2026</v>
       </c>
-      <c r="D472" s="2">
+      <c r="D472" s="1">
         <v>46175</v>
       </c>
       <c r="G472" t="s">
@@ -23886,7 +23860,7 @@
       <c r="C473">
         <v>2026</v>
       </c>
-      <c r="D473" s="2">
+      <c r="D473" s="1">
         <v>46175</v>
       </c>
       <c r="G473" t="s">
@@ -23924,7 +23898,7 @@
       <c r="C474">
         <v>2026</v>
       </c>
-      <c r="D474" s="2">
+      <c r="D474" s="1">
         <v>46175</v>
       </c>
       <c r="G474" t="s">
@@ -23962,7 +23936,7 @@
       <c r="C475">
         <v>2026</v>
       </c>
-      <c r="D475" s="2">
+      <c r="D475" s="1">
         <v>46230</v>
       </c>
       <c r="F475" t="s">
@@ -24035,7 +24009,7 @@
       <c r="C477">
         <v>2026</v>
       </c>
-      <c r="D477" s="2">
+      <c r="D477" s="1">
         <v>46209</v>
       </c>
       <c r="F477" t="s">
@@ -24207,7 +24181,7 @@
       <c r="C482">
         <v>2026</v>
       </c>
-      <c r="D482" s="2">
+      <c r="D482" s="1">
         <v>46230</v>
       </c>
       <c r="F482" t="s">
@@ -24248,7 +24222,7 @@
       <c r="C483">
         <v>2026</v>
       </c>
-      <c r="D483" s="2">
+      <c r="D483" s="1">
         <v>46230</v>
       </c>
       <c r="F483" t="s">
@@ -24289,7 +24263,7 @@
       <c r="C484">
         <v>2026</v>
       </c>
-      <c r="D484" s="2">
+      <c r="D484" s="1">
         <v>46230</v>
       </c>
       <c r="F484" t="s">
@@ -24554,7 +24528,7 @@
       <c r="C492">
         <v>2026</v>
       </c>
-      <c r="D492" s="2">
+      <c r="D492" s="1">
         <v>46230</v>
       </c>
       <c r="F492" t="s">
@@ -24595,7 +24569,7 @@
       <c r="C493">
         <v>2026</v>
       </c>
-      <c r="D493" s="2">
+      <c r="D493" s="1">
         <v>46230</v>
       </c>
       <c r="F493" t="s">
@@ -24700,7 +24674,7 @@
       <c r="C496">
         <v>2026</v>
       </c>
-      <c r="D496" s="2">
+      <c r="D496" s="1">
         <v>46230</v>
       </c>
       <c r="F496" t="s">
@@ -24744,7 +24718,7 @@
       <c r="C497">
         <v>2026</v>
       </c>
-      <c r="D497" s="2">
+      <c r="D497" s="1">
         <v>46230</v>
       </c>
       <c r="F497" t="s">
@@ -24785,7 +24759,7 @@
       <c r="C498">
         <v>2026</v>
       </c>
-      <c r="D498" s="2">
+      <c r="D498" s="1">
         <v>46157</v>
       </c>
       <c r="G498" t="s">
@@ -24823,7 +24797,7 @@
       <c r="C499">
         <v>2026</v>
       </c>
-      <c r="D499" s="2">
+      <c r="D499" s="1">
         <v>46213</v>
       </c>
       <c r="F499" t="s">
@@ -24899,7 +24873,7 @@
       <c r="C501">
         <v>2026</v>
       </c>
-      <c r="D501" s="2">
+      <c r="D501" s="1">
         <v>46205</v>
       </c>
       <c r="F501" t="s">
@@ -24943,7 +24917,7 @@
       <c r="C502">
         <v>2026</v>
       </c>
-      <c r="D502" s="2">
+      <c r="D502" s="1">
         <v>46176</v>
       </c>
       <c r="F502" t="s">
@@ -24984,7 +24958,7 @@
       <c r="C503">
         <v>2026</v>
       </c>
-      <c r="D503" s="2">
+      <c r="D503" s="1">
         <v>46150</v>
       </c>
       <c r="F503" t="s">
@@ -25089,7 +25063,7 @@
       <c r="C506">
         <v>2026</v>
       </c>
-      <c r="D506" s="2">
+      <c r="D506" s="1">
         <v>46220</v>
       </c>
       <c r="F506" t="s">
@@ -25133,7 +25107,7 @@
       <c r="C507">
         <v>2026</v>
       </c>
-      <c r="D507" s="2">
+      <c r="D507" s="1">
         <v>46224</v>
       </c>
       <c r="F507" t="s">
@@ -25209,7 +25183,7 @@
       <c r="C509">
         <v>2026</v>
       </c>
-      <c r="D509" s="2">
+      <c r="D509" s="1">
         <v>46155</v>
       </c>
       <c r="H509" t="s">
@@ -25244,7 +25218,7 @@
       <c r="C510">
         <v>2026</v>
       </c>
-      <c r="D510" s="2">
+      <c r="D510" s="1">
         <v>46156</v>
       </c>
       <c r="F510" t="s">
@@ -25285,7 +25259,7 @@
       <c r="C511">
         <v>2026</v>
       </c>
-      <c r="D511" s="2">
+      <c r="D511" s="1">
         <v>46185</v>
       </c>
       <c r="H511" t="s">
@@ -25320,7 +25294,7 @@
       <c r="C512">
         <v>2026</v>
       </c>
-      <c r="D512" s="2">
+      <c r="D512" s="1">
         <v>46230</v>
       </c>
       <c r="F512" t="s">
@@ -25361,7 +25335,7 @@
       <c r="C513">
         <v>2026</v>
       </c>
-      <c r="D513" s="2">
+      <c r="D513" s="1">
         <v>46230</v>
       </c>
       <c r="F513" t="s">
@@ -25402,7 +25376,7 @@
       <c r="C514">
         <v>2026</v>
       </c>
-      <c r="D514" s="2">
+      <c r="D514" s="1">
         <v>46230</v>
       </c>
       <c r="F514" t="s">
@@ -25443,7 +25417,7 @@
       <c r="C515">
         <v>2026</v>
       </c>
-      <c r="D515" s="2">
+      <c r="D515" s="1">
         <v>46230</v>
       </c>
       <c r="F515" t="s">
@@ -25484,7 +25458,7 @@
       <c r="C516">
         <v>2026</v>
       </c>
-      <c r="D516" s="2">
+      <c r="D516" s="1">
         <v>46230</v>
       </c>
       <c r="F516" t="s">
@@ -25589,7 +25563,7 @@
       <c r="C519">
         <v>2026</v>
       </c>
-      <c r="D519" s="2">
+      <c r="D519" s="1">
         <v>46147</v>
       </c>
       <c r="G519" t="s">
@@ -25723,7 +25697,7 @@
       <c r="C523">
         <v>2026</v>
       </c>
-      <c r="D523" s="2">
+      <c r="D523" s="1">
         <v>46164</v>
       </c>
       <c r="F523" t="s">
@@ -25860,7 +25834,7 @@
       <c r="C527">
         <v>2026</v>
       </c>
-      <c r="D527" s="2">
+      <c r="D527" s="1">
         <v>46230</v>
       </c>
       <c r="F527" t="s">
@@ -25997,7 +25971,7 @@
       <c r="C531">
         <v>2026</v>
       </c>
-      <c r="D531" s="2">
+      <c r="D531" s="1">
         <v>46171</v>
       </c>
       <c r="F531" t="s">
@@ -26102,7 +26076,7 @@
       <c r="C534">
         <v>2026</v>
       </c>
-      <c r="D534" s="2">
+      <c r="D534" s="1">
         <v>46176</v>
       </c>
       <c r="G534" t="s">
@@ -26140,7 +26114,7 @@
       <c r="C535">
         <v>2026</v>
       </c>
-      <c r="D535" s="2">
+      <c r="D535" s="1">
         <v>46230</v>
       </c>
       <c r="F535" t="s">
@@ -26341,7 +26315,7 @@
       <c r="C541">
         <v>2026</v>
       </c>
-      <c r="D541" s="2">
+      <c r="D541" s="1">
         <v>46211</v>
       </c>
       <c r="F541" t="s">
@@ -26385,7 +26359,7 @@
       <c r="C542">
         <v>2026</v>
       </c>
-      <c r="D542" s="2">
+      <c r="D542" s="1">
         <v>46183</v>
       </c>
       <c r="H542" t="s">
@@ -26420,7 +26394,7 @@
       <c r="C543">
         <v>2026</v>
       </c>
-      <c r="D543" s="2">
+      <c r="D543" s="1">
         <v>46191</v>
       </c>
       <c r="H543" t="s">
@@ -26455,7 +26429,7 @@
       <c r="C544">
         <v>2026</v>
       </c>
-      <c r="D544" s="2">
+      <c r="D544" s="1">
         <v>46191</v>
       </c>
       <c r="G544" t="s">
@@ -26653,7 +26627,7 @@
       <c r="C550">
         <v>2026</v>
       </c>
-      <c r="D550" s="2">
+      <c r="D550" s="1">
         <v>46230</v>
       </c>
       <c r="F550" t="s">
@@ -26758,7 +26732,7 @@
       <c r="C553">
         <v>2026</v>
       </c>
-      <c r="D553" s="2">
+      <c r="D553" s="1">
         <v>46230</v>
       </c>
       <c r="F553" t="s">
@@ -26799,7 +26773,7 @@
       <c r="C554">
         <v>2026</v>
       </c>
-      <c r="D554" s="2">
+      <c r="D554" s="1">
         <v>46191</v>
       </c>
       <c r="G554" t="s">
@@ -26965,7 +26939,7 @@
       <c r="C559">
         <v>2026</v>
       </c>
-      <c r="D559" s="2">
+      <c r="D559" s="1">
         <v>46191</v>
       </c>
       <c r="G559" t="s">
@@ -27163,7 +27137,7 @@
       <c r="C565">
         <v>2026</v>
       </c>
-      <c r="D565" s="2">
+      <c r="D565" s="1">
         <v>46230</v>
       </c>
       <c r="F565" t="s">
@@ -27783,7 +27757,7 @@
       <c r="C584">
         <v>2026</v>
       </c>
-      <c r="D584" s="2">
+      <c r="D584" s="1">
         <v>46226</v>
       </c>
       <c r="F584" t="s">
@@ -28307,7 +28281,7 @@
       <c r="C600">
         <v>2026</v>
       </c>
-      <c r="D600" s="2">
+      <c r="D600" s="1">
         <v>45802</v>
       </c>
       <c r="F600" t="s">
@@ -28351,7 +28325,7 @@
       <c r="C601">
         <v>2026</v>
       </c>
-      <c r="D601" s="2">
+      <c r="D601" s="1">
         <v>45860</v>
       </c>
       <c r="F601" t="s">
@@ -28392,7 +28366,7 @@
       <c r="C602">
         <v>2026</v>
       </c>
-      <c r="D602" s="2">
+      <c r="D602" s="1">
         <v>45860</v>
       </c>
       <c r="H602" t="s">
@@ -28427,7 +28401,7 @@
       <c r="C603">
         <v>2026</v>
       </c>
-      <c r="D603" s="2">
+      <c r="D603" s="1">
         <v>45856</v>
       </c>
       <c r="F603" t="s">
@@ -28468,7 +28442,7 @@
       <c r="C604">
         <v>2026</v>
       </c>
-      <c r="D604" s="2">
+      <c r="D604" s="1">
         <v>46101</v>
       </c>
       <c r="F604" t="s">
@@ -28509,7 +28483,7 @@
       <c r="C605">
         <v>2026</v>
       </c>
-      <c r="D605" s="2">
+      <c r="D605" s="1">
         <v>46101</v>
       </c>
       <c r="F605" t="s">
@@ -28550,7 +28524,7 @@
       <c r="C606">
         <v>2026</v>
       </c>
-      <c r="D606" s="2">
+      <c r="D606" s="1">
         <v>45863</v>
       </c>
       <c r="F606" t="s">
@@ -28591,7 +28565,7 @@
       <c r="C607">
         <v>2026</v>
       </c>
-      <c r="D607" s="2">
+      <c r="D607" s="1">
         <v>45863</v>
       </c>
       <c r="F607" t="s">
@@ -28632,7 +28606,7 @@
       <c r="C608">
         <v>2026</v>
       </c>
-      <c r="D608" s="2">
+      <c r="D608" s="1">
         <v>46086</v>
       </c>
       <c r="F608" t="s">
@@ -28673,7 +28647,7 @@
       <c r="C609">
         <v>2026</v>
       </c>
-      <c r="D609" s="2">
+      <c r="D609" s="1">
         <v>45874</v>
       </c>
       <c r="F609" t="s">
@@ -28714,7 +28688,7 @@
       <c r="C610">
         <v>2026</v>
       </c>
-      <c r="D610" s="2">
+      <c r="D610" s="1">
         <v>45894</v>
       </c>
       <c r="F610" t="s">
@@ -28755,7 +28729,7 @@
       <c r="C611">
         <v>2026</v>
       </c>
-      <c r="D611" s="2">
+      <c r="D611" s="1">
         <v>45894</v>
       </c>
       <c r="F611" t="s">
@@ -28796,7 +28770,7 @@
       <c r="C612">
         <v>2026</v>
       </c>
-      <c r="D612" s="2">
+      <c r="D612" s="1">
         <v>46119</v>
       </c>
       <c r="F612" t="s">
@@ -28837,7 +28811,7 @@
       <c r="C613">
         <v>2026</v>
       </c>
-      <c r="D613" s="2">
+      <c r="D613" s="1">
         <v>45898</v>
       </c>
       <c r="F613" t="s">
@@ -28878,7 +28852,7 @@
       <c r="C614">
         <v>2026</v>
       </c>
-      <c r="D614" s="2">
+      <c r="D614" s="1">
         <v>45971</v>
       </c>
       <c r="F614" t="s">
@@ -28919,7 +28893,7 @@
       <c r="C615">
         <v>2026</v>
       </c>
-      <c r="D615" s="2">
+      <c r="D615" s="1">
         <v>46119</v>
       </c>
       <c r="F615" t="s">
@@ -28960,7 +28934,7 @@
       <c r="C616">
         <v>2026</v>
       </c>
-      <c r="D616" s="2">
+      <c r="D616" s="1">
         <v>46092</v>
       </c>
       <c r="F616" t="s">
@@ -29001,7 +28975,7 @@
       <c r="C617">
         <v>2026</v>
       </c>
-      <c r="D617" s="2">
+      <c r="D617" s="1">
         <v>46119</v>
       </c>
       <c r="F617" t="s">
@@ -29042,7 +29016,7 @@
       <c r="C618">
         <v>2026</v>
       </c>
-      <c r="D618" s="2">
+      <c r="D618" s="1">
         <v>46029</v>
       </c>
       <c r="F618" t="s">
@@ -29083,7 +29057,7 @@
       <c r="C619">
         <v>2026</v>
       </c>
-      <c r="D619" s="2">
+      <c r="D619" s="1">
         <v>46029</v>
       </c>
       <c r="F619" t="s">
@@ -29124,7 +29098,7 @@
       <c r="C620">
         <v>2026</v>
       </c>
-      <c r="D620" s="2">
+      <c r="D620" s="1">
         <v>46063</v>
       </c>
       <c r="H620" t="s">
@@ -29159,7 +29133,7 @@
       <c r="C621">
         <v>2026</v>
       </c>
-      <c r="D621" s="2">
+      <c r="D621" s="1">
         <v>46232</v>
       </c>
       <c r="G621" t="s">
@@ -29197,7 +29171,7 @@
       <c r="C622">
         <v>2026</v>
       </c>
-      <c r="D622" s="2">
+      <c r="D622" s="1">
         <v>46232</v>
       </c>
       <c r="G622" t="s">
@@ -29235,7 +29209,7 @@
       <c r="C623">
         <v>2026</v>
       </c>
-      <c r="D623" s="2">
+      <c r="D623" s="1">
         <v>46232</v>
       </c>
       <c r="G623" t="s">
@@ -29273,7 +29247,7 @@
       <c r="C624">
         <v>2026</v>
       </c>
-      <c r="D624" s="2">
+      <c r="D624" s="1">
         <v>46232</v>
       </c>
       <c r="G624" t="s">
@@ -29311,7 +29285,7 @@
       <c r="C625">
         <v>2026</v>
       </c>
-      <c r="D625" s="2">
+      <c r="D625" s="1">
         <v>46155</v>
       </c>
       <c r="H625" t="s">
@@ -29346,7 +29320,7 @@
       <c r="C626">
         <v>2026</v>
       </c>
-      <c r="D626" s="2">
+      <c r="D626" s="1">
         <v>46139</v>
       </c>
       <c r="F626" t="s">
@@ -29387,7 +29361,7 @@
       <c r="C627">
         <v>2026</v>
       </c>
-      <c r="D627" s="2">
+      <c r="D627" s="1">
         <v>46155</v>
       </c>
       <c r="F627" t="s">
@@ -29428,7 +29402,7 @@
       <c r="C628">
         <v>2026</v>
       </c>
-      <c r="D628" s="2">
+      <c r="D628" s="1">
         <v>46155</v>
       </c>
       <c r="H628" t="s">
@@ -29463,7 +29437,7 @@
       <c r="C629">
         <v>2026</v>
       </c>
-      <c r="D629" s="2">
+      <c r="D629" s="1">
         <v>46147</v>
       </c>
       <c r="H629" t="s">
@@ -29498,7 +29472,7 @@
       <c r="C630">
         <v>2026</v>
       </c>
-      <c r="D630" s="2">
+      <c r="D630" s="1">
         <v>46164</v>
       </c>
       <c r="F630" t="s">
@@ -29539,7 +29513,7 @@
       <c r="C631">
         <v>2026</v>
       </c>
-      <c r="D631" s="2">
+      <c r="D631" s="1">
         <v>46225</v>
       </c>
       <c r="F631" t="s">
@@ -29580,7 +29554,7 @@
       <c r="C632">
         <v>2026</v>
       </c>
-      <c r="D632" s="2">
+      <c r="D632" s="1">
         <v>46225</v>
       </c>
       <c r="F632" t="s">
@@ -29621,7 +29595,7 @@
       <c r="C633">
         <v>2026</v>
       </c>
-      <c r="D633" s="2">
+      <c r="D633" s="1">
         <v>46225</v>
       </c>
       <c r="F633" t="s">
@@ -29662,7 +29636,7 @@
       <c r="C634">
         <v>2026</v>
       </c>
-      <c r="D634" s="2">
+      <c r="D634" s="1">
         <v>46248</v>
       </c>
       <c r="H634" t="s">
@@ -29697,7 +29671,7 @@
       <c r="C635">
         <v>2026</v>
       </c>
-      <c r="D635" s="2">
+      <c r="D635" s="1">
         <v>46248</v>
       </c>
       <c r="F635" t="s">
@@ -29738,7 +29712,7 @@
       <c r="C636">
         <v>2026</v>
       </c>
-      <c r="D636" s="2">
+      <c r="D636" s="1">
         <v>46171</v>
       </c>
       <c r="H636" t="s">
@@ -29773,7 +29747,7 @@
       <c r="C637">
         <v>2026</v>
       </c>
-      <c r="D637" s="2">
+      <c r="D637" s="1">
         <v>46176</v>
       </c>
       <c r="H637" t="s">
@@ -29808,7 +29782,7 @@
       <c r="C638">
         <v>2026</v>
       </c>
-      <c r="D638" s="2">
+      <c r="D638" s="1">
         <v>46225</v>
       </c>
       <c r="F638" t="s">
@@ -29849,7 +29823,7 @@
       <c r="C639">
         <v>2026</v>
       </c>
-      <c r="D639" s="2">
+      <c r="D639" s="1">
         <v>46211</v>
       </c>
       <c r="H639" t="s">
@@ -29884,7 +29858,7 @@
       <c r="C640">
         <v>2026</v>
       </c>
-      <c r="D640" s="2">
+      <c r="D640" s="1">
         <v>46183</v>
       </c>
       <c r="H640" t="s">
@@ -29919,7 +29893,7 @@
       <c r="C641">
         <v>2026</v>
       </c>
-      <c r="D641" s="2">
+      <c r="D641" s="1">
         <v>46191</v>
       </c>
       <c r="F641" t="s">
@@ -29960,7 +29934,7 @@
       <c r="C642">
         <v>2026</v>
       </c>
-      <c r="D642" s="2">
+      <c r="D642" s="1">
         <v>46176</v>
       </c>
       <c r="H642" t="s">
@@ -29995,7 +29969,7 @@
       <c r="C643">
         <v>2026</v>
       </c>
-      <c r="D643" s="2">
+      <c r="D643" s="1">
         <v>46191</v>
       </c>
       <c r="H643" t="s">
@@ -30030,7 +30004,7 @@
       <c r="C644">
         <v>2026</v>
       </c>
-      <c r="D644" s="2">
+      <c r="D644" s="1">
         <v>46241</v>
       </c>
       <c r="F644" t="s">
@@ -30074,7 +30048,7 @@
       <c r="C645">
         <v>2026</v>
       </c>
-      <c r="D645" s="2">
+      <c r="D645" s="1">
         <v>46191</v>
       </c>
       <c r="F645" t="s">
@@ -30115,7 +30089,7 @@
       <c r="C646">
         <v>2026</v>
       </c>
-      <c r="D646" s="2">
+      <c r="D646" s="1">
         <v>46191</v>
       </c>
       <c r="F646" t="s">
@@ -30156,7 +30130,7 @@
       <c r="C647">
         <v>2026</v>
       </c>
-      <c r="D647" s="2">
+      <c r="D647" s="1">
         <v>46191</v>
       </c>
       <c r="H647" t="s">
@@ -30191,7 +30165,7 @@
       <c r="C648">
         <v>2026</v>
       </c>
-      <c r="D648" s="2">
+      <c r="D648" s="1">
         <v>46241</v>
       </c>
       <c r="F648" t="s">
@@ -30232,7 +30206,7 @@
       <c r="C649">
         <v>2026</v>
       </c>
-      <c r="D649" s="2">
+      <c r="D649" s="1">
         <v>46191</v>
       </c>
       <c r="H649" t="s">
@@ -30267,7 +30241,7 @@
       <c r="C650">
         <v>2026</v>
       </c>
-      <c r="D650" s="2">
+      <c r="D650" s="1">
         <v>46248</v>
       </c>
       <c r="H650" t="s">
@@ -30302,7 +30276,7 @@
       <c r="C651">
         <v>2026</v>
       </c>
-      <c r="D651" s="2">
+      <c r="D651" s="1">
         <v>46241</v>
       </c>
       <c r="F651" t="s">
@@ -30343,7 +30317,7 @@
       <c r="C652">
         <v>2026</v>
       </c>
-      <c r="D652" s="2">
+      <c r="D652" s="1">
         <v>46241</v>
       </c>
       <c r="F652" t="s">
@@ -30384,7 +30358,7 @@
       <c r="C653">
         <v>2026</v>
       </c>
-      <c r="D653" s="2">
+      <c r="D653" s="1">
         <v>46225</v>
       </c>
       <c r="F653" t="s">
@@ -30425,7 +30399,7 @@
       <c r="C654">
         <v>2026</v>
       </c>
-      <c r="D654" s="2">
+      <c r="D654" s="1">
         <v>46241</v>
       </c>
       <c r="F654" t="s">
@@ -30466,7 +30440,7 @@
       <c r="C655">
         <v>2026</v>
       </c>
-      <c r="D655" s="2">
+      <c r="D655" s="1">
         <v>46241</v>
       </c>
       <c r="F655" t="s">
@@ -30507,7 +30481,7 @@
       <c r="C656">
         <v>2026</v>
       </c>
-      <c r="D656" s="2">
+      <c r="D656" s="1">
         <v>46241</v>
       </c>
       <c r="F656" t="s">
@@ -30548,7 +30522,7 @@
       <c r="C657">
         <v>2026</v>
       </c>
-      <c r="D657" s="2">
+      <c r="D657" s="1">
         <v>46248</v>
       </c>
       <c r="H657" t="s">
@@ -30583,7 +30557,7 @@
       <c r="C658">
         <v>2026</v>
       </c>
-      <c r="D658" s="2">
+      <c r="D658" s="1">
         <v>46248</v>
       </c>
       <c r="H658" t="s">
@@ -30618,7 +30592,7 @@
       <c r="C659">
         <v>2026</v>
       </c>
-      <c r="D659" s="2">
+      <c r="D659" s="1">
         <v>46248</v>
       </c>
       <c r="F659" t="s">
@@ -30659,7 +30633,7 @@
       <c r="C660">
         <v>2026</v>
       </c>
-      <c r="D660" s="2">
+      <c r="D660" s="1">
         <v>46248</v>
       </c>
       <c r="F660" t="s">
@@ -30700,7 +30674,7 @@
       <c r="C661">
         <v>2026</v>
       </c>
-      <c r="D661" s="2">
+      <c r="D661" s="1">
         <v>46248</v>
       </c>
       <c r="F661" t="s">
@@ -30741,7 +30715,7 @@
       <c r="C662">
         <v>2026</v>
       </c>
-      <c r="D662" s="2">
+      <c r="D662" s="1">
         <v>45989</v>
       </c>
       <c r="G662" t="s">
@@ -30779,7 +30753,7 @@
       <c r="C663">
         <v>2026</v>
       </c>
-      <c r="D663" s="2">
+      <c r="D663" s="1">
         <v>46002</v>
       </c>
       <c r="G663" t="s">
@@ -30817,7 +30791,7 @@
       <c r="C664">
         <v>2026</v>
       </c>
-      <c r="D664" s="2">
+      <c r="D664" s="1">
         <v>46002</v>
       </c>
       <c r="G664" t="s">
@@ -30855,7 +30829,7 @@
       <c r="C665">
         <v>2026</v>
       </c>
-      <c r="D665" s="2">
+      <c r="D665" s="1">
         <v>46225</v>
       </c>
       <c r="F665" t="s">
@@ -30896,7 +30870,7 @@
       <c r="C666">
         <v>2026</v>
       </c>
-      <c r="D666" s="2">
+      <c r="D666" s="1">
         <v>46211</v>
       </c>
       <c r="F666" t="s">
@@ -30937,7 +30911,7 @@
       <c r="C667">
         <v>2026</v>
       </c>
-      <c r="D667" s="2">
+      <c r="D667" s="1">
         <v>46248</v>
       </c>
       <c r="F667" t="s">
@@ -30978,7 +30952,7 @@
       <c r="C668">
         <v>2026</v>
       </c>
-      <c r="D668" s="2">
+      <c r="D668" s="1">
         <v>46248</v>
       </c>
       <c r="F668" t="s">
@@ -31051,7 +31025,7 @@
       <c r="C670">
         <v>2026</v>
       </c>
-      <c r="D670" s="2">
+      <c r="D670" s="1">
         <v>46255</v>
       </c>
       <c r="F670" t="s">
@@ -31252,7 +31226,7 @@
       <c r="C676">
         <v>2026</v>
       </c>
-      <c r="D676" s="2">
+      <c r="D676" s="1">
         <v>46265</v>
       </c>
       <c r="H676" t="s">
@@ -31287,7 +31261,7 @@
       <c r="C677">
         <v>2026</v>
       </c>
-      <c r="D677" s="2">
+      <c r="D677" s="1">
         <v>46265</v>
       </c>
       <c r="H677" t="s">
@@ -31322,7 +31296,7 @@
       <c r="C678">
         <v>2026</v>
       </c>
-      <c r="D678" s="2">
+      <c r="D678" s="1">
         <v>46265</v>
       </c>
       <c r="H678" t="s">
@@ -31677,7 +31651,7 @@
       <c r="C689">
         <v>2026</v>
       </c>
-      <c r="D689" s="2">
+      <c r="D689" s="1">
         <v>46265</v>
       </c>
       <c r="H689" t="s">
@@ -31712,7 +31686,7 @@
       <c r="C690">
         <v>2026</v>
       </c>
-      <c r="D690" s="2">
+      <c r="D690" s="1">
         <v>46265</v>
       </c>
       <c r="H690" t="s">

</xml_diff>